<commit_message>
fix(product): correct cancelled visit balances and preserve sample formulas
</commit_message>
<xml_diff>
--- a/commercial/beachheads/pet-sitting-operations-tracker/Pet-Sitting-Business-Operations-Tracker.xlsx
+++ b/commercial/beachheads/pet-sitting-operations-tracker/Pet-Sitting-Business-Operations-Tracker.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rf13cb9225e884f24"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Visits" sheetId="2" r:id="R58f1dfd7cc114141"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Clients &amp; Pets" sheetId="3" r:id="R2c3d62eb79ab446a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Expenses" sheetId="4" r:id="Rc6768f48e4c24fc0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Services" sheetId="5" r:id="R83d6773a2ee14db3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide &amp; Sources" sheetId="6" r:id="R682351ad1d84459a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R6d24a5f3ed2e4125"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Visits" sheetId="2" r:id="Rb77ce8afab8140d7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Clients &amp; Pets" sheetId="3" r:id="Rcb65afba69444ae2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Expenses" sheetId="4" r:id="Rd2c070508fee4ff5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Services" sheetId="5" r:id="R612893a7efe14f92"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide &amp; Sources" sheetId="6" r:id="Ra71b484616404e24"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -535,7 +535,7 @@
         <x:color rgb="FF166534"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE7F4EA"/>
         </x:patternFill>
       </x:fill>
@@ -545,7 +545,7 @@
         <x:color rgb="FF991B1B"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFDECEC"/>
         </x:patternFill>
       </x:fill>
@@ -556,7 +556,7 @@
         <x:color rgb="FF991B1B"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFDECEC"/>
         </x:patternFill>
       </x:fill>
@@ -566,7 +566,7 @@
         <x:color rgb="FF92400E"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF3CD"/>
         </x:patternFill>
       </x:fill>
@@ -1015,7 +1015,7 @@
       </x:c>
       <x:c r="F6" s="2"/>
       <x:c r="G6" s="2" t="str">
-        <x:v>Mileage estimate / mile</x:v>
+        <x:v>Rate per mile</x:v>
       </x:c>
       <x:c r="H6" s="10" t="n">
         <x:v>0.7</x:v>
@@ -4598,11 +4598,11 @@
         <x:v>28</x:v>
       </x:c>
       <x:c r="J7" s="62" t="n">
-        <x:f>IF(A7="","",MAX(0,H7-I7))</x:f>
+        <x:f>IF(A7="","",IF(G7="Cancelled",0,MAX(0,H7-I7)))</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="K7" s="2" t="str">
-        <x:f>IF(A7="","",IF(J7=0,"Paid",IF(I7=0,"Unpaid","Partial")))</x:f>
+        <x:f>IF(A7="","",IF(G7="Cancelled","No charge",IF(J7=0,"Paid",IF(I7&gt;0,"Partial","Unpaid"))))</x:f>
         <x:v>Paid</x:v>
       </x:c>
       <x:c r="L7" s="2" t="str">
@@ -4654,11 +4654,11 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="J8" s="62" t="n">
-        <x:f>IF(A8="","",MAX(0,H8-I8))</x:f>
+        <x:f>IF(A8="","",IF(G8="Cancelled",0,MAX(0,H8-I8)))</x:f>
         <x:v>20</x:v>
       </x:c>
       <x:c r="K8" s="2" t="str">
-        <x:f>IF(A8="","",IF(J8=0,"Paid",IF(I8=0,"Unpaid","Partial")))</x:f>
+        <x:f>IF(A8="","",IF(G8="Cancelled","No charge",IF(J8=0,"Paid",IF(I8&gt;0,"Partial","Unpaid"))))</x:f>
         <x:v>Partial</x:v>
       </x:c>
       <x:c r="L8" s="2" t="str">
@@ -4711,11 +4711,11 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="J9" s="62" t="n">
-        <x:f>IF(A9="","",MAX(0,H9-I9))</x:f>
+        <x:f>IF(A9="","",IF(G9="Cancelled",0,MAX(0,H9-I9)))</x:f>
         <x:v>28</x:v>
       </x:c>
       <x:c r="K9" s="2" t="str">
-        <x:f>IF(A9="","",IF(J9=0,"Paid",IF(I9=0,"Unpaid","Partial")))</x:f>
+        <x:f>IF(A9="","",IF(G9="Cancelled","No charge",IF(J9=0,"Paid",IF(I9&gt;0,"Partial","Unpaid"))))</x:f>
         <x:v>Unpaid</x:v>
       </x:c>
       <x:c r="L9" s="2" t="str">
@@ -4767,12 +4767,12 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="J10" s="62" t="n">
-        <x:f>IF(A10="","",MAX(0,H10-I10))</x:f>
-        <x:v>45</x:v>
+        <x:f>IF(A10="","",IF(G10="Cancelled",0,MAX(0,H10-I10)))</x:f>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="K10" s="2" t="str">
-        <x:f>IF(A10="","",IF(J10=0,"Paid",IF(I10=0,"Unpaid","Partial")))</x:f>
-        <x:v>Unpaid</x:v>
+        <x:f>IF(A10="","",IF(G10="Cancelled","No charge",IF(J10=0,"Paid",IF(I10&gt;0,"Partial","Unpaid"))))</x:f>
+        <x:v>No charge</x:v>
       </x:c>
       <x:c r="L10" s="2" t="str">
         <x:f>IF(A10="","",IF(AND(G10="Completed",J10&gt;0),"Collect balance",IF(AND(G10="Scheduled",B10&lt;TODAY()),"Review overdue visit","")))</x:f>
@@ -4805,10 +4805,10 @@
       <x:c r="H11" s="63"/>
       <x:c r="I11" s="64"/>
       <x:c r="J11" s="62" t="str">
-        <x:f>IF(A11="","",MAX(0,H11-I11))</x:f>
+        <x:f>IF(A11="","",IF(G11="Cancelled",0,MAX(0,H11-I11)))</x:f>
       </x:c>
       <x:c r="K11" s="2" t="str">
-        <x:f>IF(A11="","",IF(J11=0,"Paid",IF(I11=0,"Unpaid","Partial")))</x:f>
+        <x:f>IF(A11="","",IF(G11="Cancelled","No charge",IF(J11=0,"Paid",IF(I11&gt;0,"Partial","Unpaid"))))</x:f>
       </x:c>
       <x:c r="L11" s="2" t="str">
         <x:f>IF(A11="","",IF(AND(G11="Completed",J11&gt;0),"Collect balance",IF(AND(G11="Scheduled",B11&lt;TODAY()),"Review overdue visit","")))</x:f>
@@ -4839,10 +4839,10 @@
       <x:c r="H12" s="63"/>
       <x:c r="I12" s="64"/>
       <x:c r="J12" s="62" t="str">
-        <x:f>IF(A12="","",MAX(0,H12-I12))</x:f>
+        <x:f>IF(A12="","",IF(G12="Cancelled",0,MAX(0,H12-I12)))</x:f>
       </x:c>
       <x:c r="K12" s="2" t="str">
-        <x:f>IF(A12="","",IF(J12=0,"Paid",IF(I12=0,"Unpaid","Partial")))</x:f>
+        <x:f>IF(A12="","",IF(G12="Cancelled","No charge",IF(J12=0,"Paid",IF(I12&gt;0,"Partial","Unpaid"))))</x:f>
       </x:c>
       <x:c r="L12" s="2" t="str">
         <x:f>IF(A12="","",IF(AND(G12="Completed",J12&gt;0),"Collect balance",IF(AND(G12="Scheduled",B12&lt;TODAY()),"Review overdue visit","")))</x:f>
@@ -4873,10 +4873,10 @@
       <x:c r="H13" s="63"/>
       <x:c r="I13" s="64"/>
       <x:c r="J13" s="62" t="str">
-        <x:f>IF(A13="","",MAX(0,H13-I13))</x:f>
+        <x:f>IF(A13="","",IF(G13="Cancelled",0,MAX(0,H13-I13)))</x:f>
       </x:c>
       <x:c r="K13" s="2" t="str">
-        <x:f>IF(A13="","",IF(J13=0,"Paid",IF(I13=0,"Unpaid","Partial")))</x:f>
+        <x:f>IF(A13="","",IF(G13="Cancelled","No charge",IF(J13=0,"Paid",IF(I13&gt;0,"Partial","Unpaid"))))</x:f>
       </x:c>
       <x:c r="L13" s="2" t="str">
         <x:f>IF(A13="","",IF(AND(G13="Completed",J13&gt;0),"Collect balance",IF(AND(G13="Scheduled",B13&lt;TODAY()),"Review overdue visit","")))</x:f>
@@ -4907,10 +4907,10 @@
       <x:c r="H14" s="63"/>
       <x:c r="I14" s="64"/>
       <x:c r="J14" s="62" t="str">
-        <x:f>IF(A14="","",MAX(0,H14-I14))</x:f>
+        <x:f>IF(A14="","",IF(G14="Cancelled",0,MAX(0,H14-I14)))</x:f>
       </x:c>
       <x:c r="K14" s="2" t="str">
-        <x:f>IF(A14="","",IF(J14=0,"Paid",IF(I14=0,"Unpaid","Partial")))</x:f>
+        <x:f>IF(A14="","",IF(G14="Cancelled","No charge",IF(J14=0,"Paid",IF(I14&gt;0,"Partial","Unpaid"))))</x:f>
       </x:c>
       <x:c r="L14" s="2" t="str">
         <x:f>IF(A14="","",IF(AND(G14="Completed",J14&gt;0),"Collect balance",IF(AND(G14="Scheduled",B14&lt;TODAY()),"Review overdue visit","")))</x:f>
@@ -4941,10 +4941,10 @@
       <x:c r="H15" s="63"/>
       <x:c r="I15" s="64"/>
       <x:c r="J15" s="62" t="str">
-        <x:f>IF(A15="","",MAX(0,H15-I15))</x:f>
+        <x:f>IF(A15="","",IF(G15="Cancelled",0,MAX(0,H15-I15)))</x:f>
       </x:c>
       <x:c r="K15" s="2" t="str">
-        <x:f>IF(A15="","",IF(J15=0,"Paid",IF(I15=0,"Unpaid","Partial")))</x:f>
+        <x:f>IF(A15="","",IF(G15="Cancelled","No charge",IF(J15=0,"Paid",IF(I15&gt;0,"Partial","Unpaid"))))</x:f>
       </x:c>
       <x:c r="L15" s="2" t="str">
         <x:f>IF(A15="","",IF(AND(G15="Completed",J15&gt;0),"Collect balance",IF(AND(G15="Scheduled",B15&lt;TODAY()),"Review overdue visit","")))</x:f>
@@ -4975,10 +4975,10 @@
       <x:c r="H16" s="63"/>
       <x:c r="I16" s="64"/>
       <x:c r="J16" s="62" t="str">
-        <x:f>IF(A16="","",MAX(0,H16-I16))</x:f>
+        <x:f>IF(A16="","",IF(G16="Cancelled",0,MAX(0,H16-I16)))</x:f>
       </x:c>
       <x:c r="K16" s="2" t="str">
-        <x:f>IF(A16="","",IF(J16=0,"Paid",IF(I16=0,"Unpaid","Partial")))</x:f>
+        <x:f>IF(A16="","",IF(G16="Cancelled","No charge",IF(J16=0,"Paid",IF(I16&gt;0,"Partial","Unpaid"))))</x:f>
       </x:c>
       <x:c r="L16" s="2" t="str">
         <x:f>IF(A16="","",IF(AND(G16="Completed",J16&gt;0),"Collect balance",IF(AND(G16="Scheduled",B16&lt;TODAY()),"Review overdue visit","")))</x:f>
@@ -5009,10 +5009,10 @@
       <x:c r="H17" s="63"/>
       <x:c r="I17" s="64"/>
       <x:c r="J17" s="62" t="str">
-        <x:f>IF(A17="","",MAX(0,H17-I17))</x:f>
+        <x:f>IF(A17="","",IF(G17="Cancelled",0,MAX(0,H17-I17)))</x:f>
       </x:c>
       <x:c r="K17" s="2" t="str">
-        <x:f>IF(A17="","",IF(J17=0,"Paid",IF(I17=0,"Unpaid","Partial")))</x:f>
+        <x:f>IF(A17="","",IF(G17="Cancelled","No charge",IF(J17=0,"Paid",IF(I17&gt;0,"Partial","Unpaid"))))</x:f>
       </x:c>
       <x:c r="L17" s="2" t="str">
         <x:f>IF(A17="","",IF(AND(G17="Completed",J17&gt;0),"Collect balance",IF(AND(G17="Scheduled",B17&lt;TODAY()),"Review overdue visit","")))</x:f>
@@ -5043,10 +5043,10 @@
       <x:c r="H18" s="63"/>
       <x:c r="I18" s="64"/>
       <x:c r="J18" s="62" t="str">
-        <x:f>IF(A18="","",MAX(0,H18-I18))</x:f>
+        <x:f>IF(A18="","",IF(G18="Cancelled",0,MAX(0,H18-I18)))</x:f>
       </x:c>
       <x:c r="K18" s="2" t="str">
-        <x:f>IF(A18="","",IF(J18=0,"Paid",IF(I18=0,"Unpaid","Partial")))</x:f>
+        <x:f>IF(A18="","",IF(G18="Cancelled","No charge",IF(J18=0,"Paid",IF(I18&gt;0,"Partial","Unpaid"))))</x:f>
       </x:c>
       <x:c r="L18" s="2" t="str">
         <x:f>IF(A18="","",IF(AND(G18="Completed",J18&gt;0),"Collect balance",IF(AND(G18="Scheduled",B18&lt;TODAY()),"Review overdue visit","")))</x:f>
@@ -5077,10 +5077,10 @@
       <x:c r="H19" s="63"/>
       <x:c r="I19" s="64"/>
       <x:c r="J19" s="62" t="str">
-        <x:f>IF(A19="","",MAX(0,H19-I19))</x:f>
+        <x:f>IF(A19="","",IF(G19="Cancelled",0,MAX(0,H19-I19)))</x:f>
       </x:c>
       <x:c r="K19" s="2" t="str">
-        <x:f>IF(A19="","",IF(J19=0,"Paid",IF(I19=0,"Unpaid","Partial")))</x:f>
+        <x:f>IF(A19="","",IF(G19="Cancelled","No charge",IF(J19=0,"Paid",IF(I19&gt;0,"Partial","Unpaid"))))</x:f>
       </x:c>
       <x:c r="L19" s="2" t="str">
         <x:f>IF(A19="","",IF(AND(G19="Completed",J19&gt;0),"Collect balance",IF(AND(G19="Scheduled",B19&lt;TODAY()),"Review overdue visit","")))</x:f>
@@ -5111,10 +5111,10 @@
       <x:c r="H20" s="63"/>
       <x:c r="I20" s="64"/>
       <x:c r="J20" s="62" t="str">
-        <x:f>IF(A20="","",MAX(0,H20-I20))</x:f>
+        <x:f>IF(A20="","",IF(G20="Cancelled",0,MAX(0,H20-I20)))</x:f>
       </x:c>
       <x:c r="K20" s="2" t="str">
-        <x:f>IF(A20="","",IF(J20=0,"Paid",IF(I20=0,"Unpaid","Partial")))</x:f>
+        <x:f>IF(A20="","",IF(G20="Cancelled","No charge",IF(J20=0,"Paid",IF(I20&gt;0,"Partial","Unpaid"))))</x:f>
       </x:c>
       <x:c r="L20" s="2" t="str">
         <x:f>IF(A20="","",IF(AND(G20="Completed",J20&gt;0),"Collect balance",IF(AND(G20="Scheduled",B20&lt;TODAY()),"Review overdue visit","")))</x:f>
@@ -5145,10 +5145,10 @@
       <x:c r="H21" s="63"/>
       <x:c r="I21" s="64"/>
       <x:c r="J21" s="62" t="str">
-        <x:f>IF(A21="","",MAX(0,H21-I21))</x:f>
+        <x:f>IF(A21="","",IF(G21="Cancelled",0,MAX(0,H21-I21)))</x:f>
       </x:c>
       <x:c r="K21" s="2" t="str">
-        <x:f>IF(A21="","",IF(J21=0,"Paid",IF(I21=0,"Unpaid","Partial")))</x:f>
+        <x:f>IF(A21="","",IF(G21="Cancelled","No charge",IF(J21=0,"Paid",IF(I21&gt;0,"Partial","Unpaid"))))</x:f>
       </x:c>
       <x:c r="L21" s="2" t="str">
         <x:f>IF(A21="","",IF(AND(G21="Completed",J21&gt;0),"Collect balance",IF(AND(G21="Scheduled",B21&lt;TODAY()),"Review overdue visit","")))</x:f>
@@ -5179,10 +5179,10 @@
       <x:c r="H22" s="63"/>
       <x:c r="I22" s="64"/>
       <x:c r="J22" s="62" t="str">
-        <x:f>IF(A22="","",MAX(0,H22-I22))</x:f>
+        <x:f>IF(A22="","",IF(G22="Cancelled",0,MAX(0,H22-I22)))</x:f>
       </x:c>
       <x:c r="K22" s="2" t="str">
-        <x:f>IF(A22="","",IF(J22=0,"Paid",IF(I22=0,"Unpaid","Partial")))</x:f>
+        <x:f>IF(A22="","",IF(G22="Cancelled","No charge",IF(J22=0,"Paid",IF(I22&gt;0,"Partial","Unpaid"))))</x:f>
       </x:c>
       <x:c r="L22" s="2" t="str">
         <x:f>IF(A22="","",IF(AND(G22="Completed",J22&gt;0),"Collect balance",IF(AND(G22="Scheduled",B22&lt;TODAY()),"Review overdue visit","")))</x:f>
@@ -5213,10 +5213,10 @@
       <x:c r="H23" s="63"/>
       <x:c r="I23" s="64"/>
       <x:c r="J23" s="62" t="str">
-        <x:f>IF(A23="","",MAX(0,H23-I23))</x:f>
+        <x:f>IF(A23="","",IF(G23="Cancelled",0,MAX(0,H23-I23)))</x:f>
       </x:c>
       <x:c r="K23" s="2" t="str">
-        <x:f>IF(A23="","",IF(J23=0,"Paid",IF(I23=0,"Unpaid","Partial")))</x:f>
+        <x:f>IF(A23="","",IF(G23="Cancelled","No charge",IF(J23=0,"Paid",IF(I23&gt;0,"Partial","Unpaid"))))</x:f>
       </x:c>
       <x:c r="L23" s="2" t="str">
         <x:f>IF(A23="","",IF(AND(G23="Completed",J23&gt;0),"Collect balance",IF(AND(G23="Scheduled",B23&lt;TODAY()),"Review overdue visit","")))</x:f>
@@ -5247,10 +5247,10 @@
       <x:c r="H24" s="63"/>
       <x:c r="I24" s="64"/>
       <x:c r="J24" s="62" t="str">
-        <x:f>IF(A24="","",MAX(0,H24-I24))</x:f>
+        <x:f>IF(A24="","",IF(G24="Cancelled",0,MAX(0,H24-I24)))</x:f>
       </x:c>
       <x:c r="K24" s="2" t="str">
-        <x:f>IF(A24="","",IF(J24=0,"Paid",IF(I24=0,"Unpaid","Partial")))</x:f>
+        <x:f>IF(A24="","",IF(G24="Cancelled","No charge",IF(J24=0,"Paid",IF(I24&gt;0,"Partial","Unpaid"))))</x:f>
       </x:c>
       <x:c r="L24" s="2" t="str">
         <x:f>IF(A24="","",IF(AND(G24="Completed",J24&gt;0),"Collect balance",IF(AND(G24="Scheduled",B24&lt;TODAY()),"Review overdue visit","")))</x:f>
@@ -5281,10 +5281,10 @@
       <x:c r="H25" s="63"/>
       <x:c r="I25" s="64"/>
       <x:c r="J25" s="62" t="str">
-        <x:f>IF(A25="","",MAX(0,H25-I25))</x:f>
+        <x:f>IF(A25="","",IF(G25="Cancelled",0,MAX(0,H25-I25)))</x:f>
       </x:c>
       <x:c r="K25" s="2" t="str">
-        <x:f>IF(A25="","",IF(J25=0,"Paid",IF(I25=0,"Unpaid","Partial")))</x:f>
+        <x:f>IF(A25="","",IF(G25="Cancelled","No charge",IF(J25=0,"Paid",IF(I25&gt;0,"Partial","Unpaid"))))</x:f>
       </x:c>
       <x:c r="L25" s="2" t="str">
         <x:f>IF(A25="","",IF(AND(G25="Completed",J25&gt;0),"Collect balance",IF(AND(G25="Scheduled",B25&lt;TODAY()),"Review overdue visit","")))</x:f>
@@ -5315,10 +5315,10 @@
       <x:c r="H26" s="63"/>
       <x:c r="I26" s="64"/>
       <x:c r="J26" s="62" t="str">
-        <x:f>IF(A26="","",MAX(0,H26-I26))</x:f>
+        <x:f>IF(A26="","",IF(G26="Cancelled",0,MAX(0,H26-I26)))</x:f>
       </x:c>
       <x:c r="K26" s="2" t="str">
-        <x:f>IF(A26="","",IF(J26=0,"Paid",IF(I26=0,"Unpaid","Partial")))</x:f>
+        <x:f>IF(A26="","",IF(G26="Cancelled","No charge",IF(J26=0,"Paid",IF(I26&gt;0,"Partial","Unpaid"))))</x:f>
       </x:c>
       <x:c r="L26" s="2" t="str">
         <x:f>IF(A26="","",IF(AND(G26="Completed",J26&gt;0),"Collect balance",IF(AND(G26="Scheduled",B26&lt;TODAY()),"Review overdue visit","")))</x:f>
@@ -5349,10 +5349,10 @@
       <x:c r="H27" s="63"/>
       <x:c r="I27" s="64"/>
       <x:c r="J27" s="62" t="str">
-        <x:f>IF(A27="","",MAX(0,H27-I27))</x:f>
+        <x:f>IF(A27="","",IF(G27="Cancelled",0,MAX(0,H27-I27)))</x:f>
       </x:c>
       <x:c r="K27" s="2" t="str">
-        <x:f>IF(A27="","",IF(J27=0,"Paid",IF(I27=0,"Unpaid","Partial")))</x:f>
+        <x:f>IF(A27="","",IF(G27="Cancelled","No charge",IF(J27=0,"Paid",IF(I27&gt;0,"Partial","Unpaid"))))</x:f>
       </x:c>
       <x:c r="L27" s="2" t="str">
         <x:f>IF(A27="","",IF(AND(G27="Completed",J27&gt;0),"Collect balance",IF(AND(G27="Scheduled",B27&lt;TODAY()),"Review overdue visit","")))</x:f>
@@ -5383,10 +5383,10 @@
       <x:c r="H28" s="63"/>
       <x:c r="I28" s="64"/>
       <x:c r="J28" s="62" t="str">
-        <x:f>IF(A28="","",MAX(0,H28-I28))</x:f>
+        <x:f>IF(A28="","",IF(G28="Cancelled",0,MAX(0,H28-I28)))</x:f>
       </x:c>
       <x:c r="K28" s="2" t="str">
-        <x:f>IF(A28="","",IF(J28=0,"Paid",IF(I28=0,"Unpaid","Partial")))</x:f>
+        <x:f>IF(A28="","",IF(G28="Cancelled","No charge",IF(J28=0,"Paid",IF(I28&gt;0,"Partial","Unpaid"))))</x:f>
       </x:c>
       <x:c r="L28" s="2" t="str">
         <x:f>IF(A28="","",IF(AND(G28="Completed",J28&gt;0),"Collect balance",IF(AND(G28="Scheduled",B28&lt;TODAY()),"Review overdue visit","")))</x:f>
@@ -5417,10 +5417,10 @@
       <x:c r="H29" s="63"/>
       <x:c r="I29" s="64"/>
       <x:c r="J29" s="62" t="str">
-        <x:f>IF(A29="","",MAX(0,H29-I29))</x:f>
+        <x:f>IF(A29="","",IF(G29="Cancelled",0,MAX(0,H29-I29)))</x:f>
       </x:c>
       <x:c r="K29" s="2" t="str">
-        <x:f>IF(A29="","",IF(J29=0,"Paid",IF(I29=0,"Unpaid","Partial")))</x:f>
+        <x:f>IF(A29="","",IF(G29="Cancelled","No charge",IF(J29=0,"Paid",IF(I29&gt;0,"Partial","Unpaid"))))</x:f>
       </x:c>
       <x:c r="L29" s="2" t="str">
         <x:f>IF(A29="","",IF(AND(G29="Completed",J29&gt;0),"Collect balance",IF(AND(G29="Scheduled",B29&lt;TODAY()),"Review overdue visit","")))</x:f>
@@ -5451,10 +5451,10 @@
       <x:c r="H30" s="63"/>
       <x:c r="I30" s="64"/>
       <x:c r="J30" s="62" t="str">
-        <x:f>IF(A30="","",MAX(0,H30-I30))</x:f>
+        <x:f>IF(A30="","",IF(G30="Cancelled",0,MAX(0,H30-I30)))</x:f>
       </x:c>
       <x:c r="K30" s="2" t="str">
-        <x:f>IF(A30="","",IF(J30=0,"Paid",IF(I30=0,"Unpaid","Partial")))</x:f>
+        <x:f>IF(A30="","",IF(G30="Cancelled","No charge",IF(J30=0,"Paid",IF(I30&gt;0,"Partial","Unpaid"))))</x:f>
       </x:c>
       <x:c r="L30" s="2" t="str">
         <x:f>IF(A30="","",IF(AND(G30="Completed",J30&gt;0),"Collect balance",IF(AND(G30="Scheduled",B30&lt;TODAY()),"Review overdue visit","")))</x:f>
@@ -5485,10 +5485,10 @@
       <x:c r="H31" s="63"/>
       <x:c r="I31" s="64"/>
       <x:c r="J31" s="62" t="str">
-        <x:f>IF(A31="","",MAX(0,H31-I31))</x:f>
+        <x:f>IF(A31="","",IF(G31="Cancelled",0,MAX(0,H31-I31)))</x:f>
       </x:c>
       <x:c r="K31" s="2" t="str">
-        <x:f>IF(A31="","",IF(J31=0,"Paid",IF(I31=0,"Unpaid","Partial")))</x:f>
+        <x:f>IF(A31="","",IF(G31="Cancelled","No charge",IF(J31=0,"Paid",IF(I31&gt;0,"Partial","Unpaid"))))</x:f>
       </x:c>
       <x:c r="L31" s="2" t="str">
         <x:f>IF(A31="","",IF(AND(G31="Completed",J31&gt;0),"Collect balance",IF(AND(G31="Scheduled",B31&lt;TODAY()),"Review overdue visit","")))</x:f>
@@ -5519,10 +5519,10 @@
       <x:c r="H32" s="63"/>
       <x:c r="I32" s="64"/>
       <x:c r="J32" s="62" t="str">
-        <x:f>IF(A32="","",MAX(0,H32-I32))</x:f>
+        <x:f>IF(A32="","",IF(G32="Cancelled",0,MAX(0,H32-I32)))</x:f>
       </x:c>
       <x:c r="K32" s="2" t="str">
-        <x:f>IF(A32="","",IF(J32=0,"Paid",IF(I32=0,"Unpaid","Partial")))</x:f>
+        <x:f>IF(A32="","",IF(G32="Cancelled","No charge",IF(J32=0,"Paid",IF(I32&gt;0,"Partial","Unpaid"))))</x:f>
       </x:c>
       <x:c r="L32" s="2" t="str">
         <x:f>IF(A32="","",IF(AND(G32="Completed",J32&gt;0),"Collect balance",IF(AND(G32="Scheduled",B32&lt;TODAY()),"Review overdue visit","")))</x:f>
@@ -5553,10 +5553,10 @@
       <x:c r="H33" s="63"/>
       <x:c r="I33" s="64"/>
       <x:c r="J33" s="62" t="str">
-        <x:f>IF(A33="","",MAX(0,H33-I33))</x:f>
+        <x:f>IF(A33="","",IF(G33="Cancelled",0,MAX(0,H33-I33)))</x:f>
       </x:c>
       <x:c r="K33" s="2" t="str">
-        <x:f>IF(A33="","",IF(J33=0,"Paid",IF(I33=0,"Unpaid","Partial")))</x:f>
+        <x:f>IF(A33="","",IF(G33="Cancelled","No charge",IF(J33=0,"Paid",IF(I33&gt;0,"Partial","Unpaid"))))</x:f>
       </x:c>
       <x:c r="L33" s="2" t="str">
         <x:f>IF(A33="","",IF(AND(G33="Completed",J33&gt;0),"Collect balance",IF(AND(G33="Scheduled",B33&lt;TODAY()),"Review overdue visit","")))</x:f>
@@ -5587,10 +5587,10 @@
       <x:c r="H34" s="63"/>
       <x:c r="I34" s="64"/>
       <x:c r="J34" s="62" t="str">
-        <x:f>IF(A34="","",MAX(0,H34-I34))</x:f>
+        <x:f>IF(A34="","",IF(G34="Cancelled",0,MAX(0,H34-I34)))</x:f>
       </x:c>
       <x:c r="K34" s="2" t="str">
-        <x:f>IF(A34="","",IF(J34=0,"Paid",IF(I34=0,"Unpaid","Partial")))</x:f>
+        <x:f>IF(A34="","",IF(G34="Cancelled","No charge",IF(J34=0,"Paid",IF(I34&gt;0,"Partial","Unpaid"))))</x:f>
       </x:c>
       <x:c r="L34" s="2" t="str">
         <x:f>IF(A34="","",IF(AND(G34="Completed",J34&gt;0),"Collect balance",IF(AND(G34="Scheduled",B34&lt;TODAY()),"Review overdue visit","")))</x:f>
@@ -5621,10 +5621,10 @@
       <x:c r="H35" s="63"/>
       <x:c r="I35" s="64"/>
       <x:c r="J35" s="62" t="str">
-        <x:f>IF(A35="","",MAX(0,H35-I35))</x:f>
+        <x:f>IF(A35="","",IF(G35="Cancelled",0,MAX(0,H35-I35)))</x:f>
       </x:c>
       <x:c r="K35" s="2" t="str">
-        <x:f>IF(A35="","",IF(J35=0,"Paid",IF(I35=0,"Unpaid","Partial")))</x:f>
+        <x:f>IF(A35="","",IF(G35="Cancelled","No charge",IF(J35=0,"Paid",IF(I35&gt;0,"Partial","Unpaid"))))</x:f>
       </x:c>
       <x:c r="L35" s="2" t="str">
         <x:f>IF(A35="","",IF(AND(G35="Completed",J35&gt;0),"Collect balance",IF(AND(G35="Scheduled",B35&lt;TODAY()),"Review overdue visit","")))</x:f>
@@ -5655,10 +5655,10 @@
       <x:c r="H36" s="63"/>
       <x:c r="I36" s="64"/>
       <x:c r="J36" s="62" t="str">
-        <x:f>IF(A36="","",MAX(0,H36-I36))</x:f>
+        <x:f>IF(A36="","",IF(G36="Cancelled",0,MAX(0,H36-I36)))</x:f>
       </x:c>
       <x:c r="K36" s="2" t="str">
-        <x:f>IF(A36="","",IF(J36=0,"Paid",IF(I36=0,"Unpaid","Partial")))</x:f>
+        <x:f>IF(A36="","",IF(G36="Cancelled","No charge",IF(J36=0,"Paid",IF(I36&gt;0,"Partial","Unpaid"))))</x:f>
       </x:c>
       <x:c r="L36" s="2" t="str">
         <x:f>IF(A36="","",IF(AND(G36="Completed",J36&gt;0),"Collect balance",IF(AND(G36="Scheduled",B36&lt;TODAY()),"Review overdue visit","")))</x:f>
@@ -5689,10 +5689,10 @@
       <x:c r="H37" s="63"/>
       <x:c r="I37" s="64"/>
       <x:c r="J37" s="62" t="str">
-        <x:f>IF(A37="","",MAX(0,H37-I37))</x:f>
+        <x:f>IF(A37="","",IF(G37="Cancelled",0,MAX(0,H37-I37)))</x:f>
       </x:c>
       <x:c r="K37" s="2" t="str">
-        <x:f>IF(A37="","",IF(J37=0,"Paid",IF(I37=0,"Unpaid","Partial")))</x:f>
+        <x:f>IF(A37="","",IF(G37="Cancelled","No charge",IF(J37=0,"Paid",IF(I37&gt;0,"Partial","Unpaid"))))</x:f>
       </x:c>
       <x:c r="L37" s="2" t="str">
         <x:f>IF(A37="","",IF(AND(G37="Completed",J37&gt;0),"Collect balance",IF(AND(G37="Scheduled",B37&lt;TODAY()),"Review overdue visit","")))</x:f>
@@ -5723,10 +5723,10 @@
       <x:c r="H38" s="63"/>
       <x:c r="I38" s="64"/>
       <x:c r="J38" s="62" t="str">
-        <x:f>IF(A38="","",MAX(0,H38-I38))</x:f>
+        <x:f>IF(A38="","",IF(G38="Cancelled",0,MAX(0,H38-I38)))</x:f>
       </x:c>
       <x:c r="K38" s="2" t="str">
-        <x:f>IF(A38="","",IF(J38=0,"Paid",IF(I38=0,"Unpaid","Partial")))</x:f>
+        <x:f>IF(A38="","",IF(G38="Cancelled","No charge",IF(J38=0,"Paid",IF(I38&gt;0,"Partial","Unpaid"))))</x:f>
       </x:c>
       <x:c r="L38" s="2" t="str">
         <x:f>IF(A38="","",IF(AND(G38="Completed",J38&gt;0),"Collect balance",IF(AND(G38="Scheduled",B38&lt;TODAY()),"Review overdue visit","")))</x:f>
@@ -5757,10 +5757,10 @@
       <x:c r="H39" s="63"/>
       <x:c r="I39" s="64"/>
       <x:c r="J39" s="62" t="str">
-        <x:f>IF(A39="","",MAX(0,H39-I39))</x:f>
+        <x:f>IF(A39="","",IF(G39="Cancelled",0,MAX(0,H39-I39)))</x:f>
       </x:c>
       <x:c r="K39" s="2" t="str">
-        <x:f>IF(A39="","",IF(J39=0,"Paid",IF(I39=0,"Unpaid","Partial")))</x:f>
+        <x:f>IF(A39="","",IF(G39="Cancelled","No charge",IF(J39=0,"Paid",IF(I39&gt;0,"Partial","Unpaid"))))</x:f>
       </x:c>
       <x:c r="L39" s="2" t="str">
         <x:f>IF(A39="","",IF(AND(G39="Completed",J39&gt;0),"Collect balance",IF(AND(G39="Scheduled",B39&lt;TODAY()),"Review overdue visit","")))</x:f>
@@ -5791,10 +5791,10 @@
       <x:c r="H40" s="63"/>
       <x:c r="I40" s="64"/>
       <x:c r="J40" s="62" t="str">
-        <x:f>IF(A40="","",MAX(0,H40-I40))</x:f>
+        <x:f>IF(A40="","",IF(G40="Cancelled",0,MAX(0,H40-I40)))</x:f>
       </x:c>
       <x:c r="K40" s="2" t="str">
-        <x:f>IF(A40="","",IF(J40=0,"Paid",IF(I40=0,"Unpaid","Partial")))</x:f>
+        <x:f>IF(A40="","",IF(G40="Cancelled","No charge",IF(J40=0,"Paid",IF(I40&gt;0,"Partial","Unpaid"))))</x:f>
       </x:c>
       <x:c r="L40" s="2" t="str">
         <x:f>IF(A40="","",IF(AND(G40="Completed",J40&gt;0),"Collect balance",IF(AND(G40="Scheduled",B40&lt;TODAY()),"Review overdue visit","")))</x:f>
@@ -5825,10 +5825,10 @@
       <x:c r="H41" s="63"/>
       <x:c r="I41" s="64"/>
       <x:c r="J41" s="62" t="str">
-        <x:f>IF(A41="","",MAX(0,H41-I41))</x:f>
+        <x:f>IF(A41="","",IF(G41="Cancelled",0,MAX(0,H41-I41)))</x:f>
       </x:c>
       <x:c r="K41" s="2" t="str">
-        <x:f>IF(A41="","",IF(J41=0,"Paid",IF(I41=0,"Unpaid","Partial")))</x:f>
+        <x:f>IF(A41="","",IF(G41="Cancelled","No charge",IF(J41=0,"Paid",IF(I41&gt;0,"Partial","Unpaid"))))</x:f>
       </x:c>
       <x:c r="L41" s="2" t="str">
         <x:f>IF(A41="","",IF(AND(G41="Completed",J41&gt;0),"Collect balance",IF(AND(G41="Scheduled",B41&lt;TODAY()),"Review overdue visit","")))</x:f>
@@ -5859,10 +5859,10 @@
       <x:c r="H42" s="63"/>
       <x:c r="I42" s="64"/>
       <x:c r="J42" s="62" t="str">
-        <x:f>IF(A42="","",MAX(0,H42-I42))</x:f>
+        <x:f>IF(A42="","",IF(G42="Cancelled",0,MAX(0,H42-I42)))</x:f>
       </x:c>
       <x:c r="K42" s="2" t="str">
-        <x:f>IF(A42="","",IF(J42=0,"Paid",IF(I42=0,"Unpaid","Partial")))</x:f>
+        <x:f>IF(A42="","",IF(G42="Cancelled","No charge",IF(J42=0,"Paid",IF(I42&gt;0,"Partial","Unpaid"))))</x:f>
       </x:c>
       <x:c r="L42" s="2" t="str">
         <x:f>IF(A42="","",IF(AND(G42="Completed",J42&gt;0),"Collect balance",IF(AND(G42="Scheduled",B42&lt;TODAY()),"Review overdue visit","")))</x:f>
@@ -5893,10 +5893,10 @@
       <x:c r="H43" s="63"/>
       <x:c r="I43" s="64"/>
       <x:c r="J43" s="62" t="str">
-        <x:f>IF(A43="","",MAX(0,H43-I43))</x:f>
+        <x:f>IF(A43="","",IF(G43="Cancelled",0,MAX(0,H43-I43)))</x:f>
       </x:c>
       <x:c r="K43" s="2" t="str">
-        <x:f>IF(A43="","",IF(J43=0,"Paid",IF(I43=0,"Unpaid","Partial")))</x:f>
+        <x:f>IF(A43="","",IF(G43="Cancelled","No charge",IF(J43=0,"Paid",IF(I43&gt;0,"Partial","Unpaid"))))</x:f>
       </x:c>
       <x:c r="L43" s="2" t="str">
         <x:f>IF(A43="","",IF(AND(G43="Completed",J43&gt;0),"Collect balance",IF(AND(G43="Scheduled",B43&lt;TODAY()),"Review overdue visit","")))</x:f>
@@ -5927,10 +5927,10 @@
       <x:c r="H44" s="63"/>
       <x:c r="I44" s="64"/>
       <x:c r="J44" s="62" t="str">
-        <x:f>IF(A44="","",MAX(0,H44-I44))</x:f>
+        <x:f>IF(A44="","",IF(G44="Cancelled",0,MAX(0,H44-I44)))</x:f>
       </x:c>
       <x:c r="K44" s="2" t="str">
-        <x:f>IF(A44="","",IF(J44=0,"Paid",IF(I44=0,"Unpaid","Partial")))</x:f>
+        <x:f>IF(A44="","",IF(G44="Cancelled","No charge",IF(J44=0,"Paid",IF(I44&gt;0,"Partial","Unpaid"))))</x:f>
       </x:c>
       <x:c r="L44" s="2" t="str">
         <x:f>IF(A44="","",IF(AND(G44="Completed",J44&gt;0),"Collect balance",IF(AND(G44="Scheduled",B44&lt;TODAY()),"Review overdue visit","")))</x:f>
@@ -5961,10 +5961,10 @@
       <x:c r="H45" s="63"/>
       <x:c r="I45" s="64"/>
       <x:c r="J45" s="62" t="str">
-        <x:f>IF(A45="","",MAX(0,H45-I45))</x:f>
+        <x:f>IF(A45="","",IF(G45="Cancelled",0,MAX(0,H45-I45)))</x:f>
       </x:c>
       <x:c r="K45" s="2" t="str">
-        <x:f>IF(A45="","",IF(J45=0,"Paid",IF(I45=0,"Unpaid","Partial")))</x:f>
+        <x:f>IF(A45="","",IF(G45="Cancelled","No charge",IF(J45=0,"Paid",IF(I45&gt;0,"Partial","Unpaid"))))</x:f>
       </x:c>
       <x:c r="L45" s="2" t="str">
         <x:f>IF(A45="","",IF(AND(G45="Completed",J45&gt;0),"Collect balance",IF(AND(G45="Scheduled",B45&lt;TODAY()),"Review overdue visit","")))</x:f>
@@ -5995,10 +5995,10 @@
       <x:c r="H46" s="63"/>
       <x:c r="I46" s="64"/>
       <x:c r="J46" s="62" t="str">
-        <x:f>IF(A46="","",MAX(0,H46-I46))</x:f>
+        <x:f>IF(A46="","",IF(G46="Cancelled",0,MAX(0,H46-I46)))</x:f>
       </x:c>
       <x:c r="K46" s="2" t="str">
-        <x:f>IF(A46="","",IF(J46=0,"Paid",IF(I46=0,"Unpaid","Partial")))</x:f>
+        <x:f>IF(A46="","",IF(G46="Cancelled","No charge",IF(J46=0,"Paid",IF(I46&gt;0,"Partial","Unpaid"))))</x:f>
       </x:c>
       <x:c r="L46" s="2" t="str">
         <x:f>IF(A46="","",IF(AND(G46="Completed",J46&gt;0),"Collect balance",IF(AND(G46="Scheduled",B46&lt;TODAY()),"Review overdue visit","")))</x:f>
@@ -6029,10 +6029,10 @@
       <x:c r="H47" s="63"/>
       <x:c r="I47" s="64"/>
       <x:c r="J47" s="62" t="str">
-        <x:f>IF(A47="","",MAX(0,H47-I47))</x:f>
+        <x:f>IF(A47="","",IF(G47="Cancelled",0,MAX(0,H47-I47)))</x:f>
       </x:c>
       <x:c r="K47" s="2" t="str">
-        <x:f>IF(A47="","",IF(J47=0,"Paid",IF(I47=0,"Unpaid","Partial")))</x:f>
+        <x:f>IF(A47="","",IF(G47="Cancelled","No charge",IF(J47=0,"Paid",IF(I47&gt;0,"Partial","Unpaid"))))</x:f>
       </x:c>
       <x:c r="L47" s="2" t="str">
         <x:f>IF(A47="","",IF(AND(G47="Completed",J47&gt;0),"Collect balance",IF(AND(G47="Scheduled",B47&lt;TODAY()),"Review overdue visit","")))</x:f>
@@ -6063,10 +6063,10 @@
       <x:c r="H48" s="63"/>
       <x:c r="I48" s="64"/>
       <x:c r="J48" s="62" t="str">
-        <x:f>IF(A48="","",MAX(0,H48-I48))</x:f>
+        <x:f>IF(A48="","",IF(G48="Cancelled",0,MAX(0,H48-I48)))</x:f>
       </x:c>
       <x:c r="K48" s="2" t="str">
-        <x:f>IF(A48="","",IF(J48=0,"Paid",IF(I48=0,"Unpaid","Partial")))</x:f>
+        <x:f>IF(A48="","",IF(G48="Cancelled","No charge",IF(J48=0,"Paid",IF(I48&gt;0,"Partial","Unpaid"))))</x:f>
       </x:c>
       <x:c r="L48" s="2" t="str">
         <x:f>IF(A48="","",IF(AND(G48="Completed",J48&gt;0),"Collect balance",IF(AND(G48="Scheduled",B48&lt;TODAY()),"Review overdue visit","")))</x:f>
@@ -6097,10 +6097,10 @@
       <x:c r="H49" s="63"/>
       <x:c r="I49" s="64"/>
       <x:c r="J49" s="62" t="str">
-        <x:f>IF(A49="","",MAX(0,H49-I49))</x:f>
+        <x:f>IF(A49="","",IF(G49="Cancelled",0,MAX(0,H49-I49)))</x:f>
       </x:c>
       <x:c r="K49" s="2" t="str">
-        <x:f>IF(A49="","",IF(J49=0,"Paid",IF(I49=0,"Unpaid","Partial")))</x:f>
+        <x:f>IF(A49="","",IF(G49="Cancelled","No charge",IF(J49=0,"Paid",IF(I49&gt;0,"Partial","Unpaid"))))</x:f>
       </x:c>
       <x:c r="L49" s="2" t="str">
         <x:f>IF(A49="","",IF(AND(G49="Completed",J49&gt;0),"Collect balance",IF(AND(G49="Scheduled",B49&lt;TODAY()),"Review overdue visit","")))</x:f>
@@ -6131,10 +6131,10 @@
       <x:c r="H50" s="63"/>
       <x:c r="I50" s="64"/>
       <x:c r="J50" s="62" t="str">
-        <x:f>IF(A50="","",MAX(0,H50-I50))</x:f>
+        <x:f>IF(A50="","",IF(G50="Cancelled",0,MAX(0,H50-I50)))</x:f>
       </x:c>
       <x:c r="K50" s="2" t="str">
-        <x:f>IF(A50="","",IF(J50=0,"Paid",IF(I50=0,"Unpaid","Partial")))</x:f>
+        <x:f>IF(A50="","",IF(G50="Cancelled","No charge",IF(J50=0,"Paid",IF(I50&gt;0,"Partial","Unpaid"))))</x:f>
       </x:c>
       <x:c r="L50" s="2" t="str">
         <x:f>IF(A50="","",IF(AND(G50="Completed",J50&gt;0),"Collect balance",IF(AND(G50="Scheduled",B50&lt;TODAY()),"Review overdue visit","")))</x:f>
@@ -6165,10 +6165,10 @@
       <x:c r="H51" s="63"/>
       <x:c r="I51" s="64"/>
       <x:c r="J51" s="62" t="str">
-        <x:f>IF(A51="","",MAX(0,H51-I51))</x:f>
+        <x:f>IF(A51="","",IF(G51="Cancelled",0,MAX(0,H51-I51)))</x:f>
       </x:c>
       <x:c r="K51" s="2" t="str">
-        <x:f>IF(A51="","",IF(J51=0,"Paid",IF(I51=0,"Unpaid","Partial")))</x:f>
+        <x:f>IF(A51="","",IF(G51="Cancelled","No charge",IF(J51=0,"Paid",IF(I51&gt;0,"Partial","Unpaid"))))</x:f>
       </x:c>
       <x:c r="L51" s="2" t="str">
         <x:f>IF(A51="","",IF(AND(G51="Completed",J51&gt;0),"Collect balance",IF(AND(G51="Scheduled",B51&lt;TODAY()),"Review overdue visit","")))</x:f>
@@ -6199,10 +6199,10 @@
       <x:c r="H52" s="63"/>
       <x:c r="I52" s="64"/>
       <x:c r="J52" s="62" t="str">
-        <x:f>IF(A52="","",MAX(0,H52-I52))</x:f>
+        <x:f>IF(A52="","",IF(G52="Cancelled",0,MAX(0,H52-I52)))</x:f>
       </x:c>
       <x:c r="K52" s="2" t="str">
-        <x:f>IF(A52="","",IF(J52=0,"Paid",IF(I52=0,"Unpaid","Partial")))</x:f>
+        <x:f>IF(A52="","",IF(G52="Cancelled","No charge",IF(J52=0,"Paid",IF(I52&gt;0,"Partial","Unpaid"))))</x:f>
       </x:c>
       <x:c r="L52" s="2" t="str">
         <x:f>IF(A52="","",IF(AND(G52="Completed",J52&gt;0),"Collect balance",IF(AND(G52="Scheduled",B52&lt;TODAY()),"Review overdue visit","")))</x:f>
@@ -6233,10 +6233,10 @@
       <x:c r="H53" s="63"/>
       <x:c r="I53" s="64"/>
       <x:c r="J53" s="62" t="str">
-        <x:f>IF(A53="","",MAX(0,H53-I53))</x:f>
+        <x:f>IF(A53="","",IF(G53="Cancelled",0,MAX(0,H53-I53)))</x:f>
       </x:c>
       <x:c r="K53" s="2" t="str">
-        <x:f>IF(A53="","",IF(J53=0,"Paid",IF(I53=0,"Unpaid","Partial")))</x:f>
+        <x:f>IF(A53="","",IF(G53="Cancelled","No charge",IF(J53=0,"Paid",IF(I53&gt;0,"Partial","Unpaid"))))</x:f>
       </x:c>
       <x:c r="L53" s="2" t="str">
         <x:f>IF(A53="","",IF(AND(G53="Completed",J53&gt;0),"Collect balance",IF(AND(G53="Scheduled",B53&lt;TODAY()),"Review overdue visit","")))</x:f>
@@ -6267,10 +6267,10 @@
       <x:c r="H54" s="63"/>
       <x:c r="I54" s="64"/>
       <x:c r="J54" s="62" t="str">
-        <x:f>IF(A54="","",MAX(0,H54-I54))</x:f>
+        <x:f>IF(A54="","",IF(G54="Cancelled",0,MAX(0,H54-I54)))</x:f>
       </x:c>
       <x:c r="K54" s="2" t="str">
-        <x:f>IF(A54="","",IF(J54=0,"Paid",IF(I54=0,"Unpaid","Partial")))</x:f>
+        <x:f>IF(A54="","",IF(G54="Cancelled","No charge",IF(J54=0,"Paid",IF(I54&gt;0,"Partial","Unpaid"))))</x:f>
       </x:c>
       <x:c r="L54" s="2" t="str">
         <x:f>IF(A54="","",IF(AND(G54="Completed",J54&gt;0),"Collect balance",IF(AND(G54="Scheduled",B54&lt;TODAY()),"Review overdue visit","")))</x:f>
@@ -6301,10 +6301,10 @@
       <x:c r="H55" s="63"/>
       <x:c r="I55" s="64"/>
       <x:c r="J55" s="62" t="str">
-        <x:f>IF(A55="","",MAX(0,H55-I55))</x:f>
+        <x:f>IF(A55="","",IF(G55="Cancelled",0,MAX(0,H55-I55)))</x:f>
       </x:c>
       <x:c r="K55" s="2" t="str">
-        <x:f>IF(A55="","",IF(J55=0,"Paid",IF(I55=0,"Unpaid","Partial")))</x:f>
+        <x:f>IF(A55="","",IF(G55="Cancelled","No charge",IF(J55=0,"Paid",IF(I55&gt;0,"Partial","Unpaid"))))</x:f>
       </x:c>
       <x:c r="L55" s="2" t="str">
         <x:f>IF(A55="","",IF(AND(G55="Completed",J55&gt;0),"Collect balance",IF(AND(G55="Scheduled",B55&lt;TODAY()),"Review overdue visit","")))</x:f>
@@ -6335,10 +6335,10 @@
       <x:c r="H56" s="63"/>
       <x:c r="I56" s="64"/>
       <x:c r="J56" s="62" t="str">
-        <x:f>IF(A56="","",MAX(0,H56-I56))</x:f>
+        <x:f>IF(A56="","",IF(G56="Cancelled",0,MAX(0,H56-I56)))</x:f>
       </x:c>
       <x:c r="K56" s="2" t="str">
-        <x:f>IF(A56="","",IF(J56=0,"Paid",IF(I56=0,"Unpaid","Partial")))</x:f>
+        <x:f>IF(A56="","",IF(G56="Cancelled","No charge",IF(J56=0,"Paid",IF(I56&gt;0,"Partial","Unpaid"))))</x:f>
       </x:c>
       <x:c r="L56" s="2" t="str">
         <x:f>IF(A56="","",IF(AND(G56="Completed",J56&gt;0),"Collect balance",IF(AND(G56="Scheduled",B56&lt;TODAY()),"Review overdue visit","")))</x:f>
@@ -6369,10 +6369,10 @@
       <x:c r="H57" s="63"/>
       <x:c r="I57" s="64"/>
       <x:c r="J57" s="62" t="str">
-        <x:f>IF(A57="","",MAX(0,H57-I57))</x:f>
+        <x:f>IF(A57="","",IF(G57="Cancelled",0,MAX(0,H57-I57)))</x:f>
       </x:c>
       <x:c r="K57" s="2" t="str">
-        <x:f>IF(A57="","",IF(J57=0,"Paid",IF(I57=0,"Unpaid","Partial")))</x:f>
+        <x:f>IF(A57="","",IF(G57="Cancelled","No charge",IF(J57=0,"Paid",IF(I57&gt;0,"Partial","Unpaid"))))</x:f>
       </x:c>
       <x:c r="L57" s="2" t="str">
         <x:f>IF(A57="","",IF(AND(G57="Completed",J57&gt;0),"Collect balance",IF(AND(G57="Scheduled",B57&lt;TODAY()),"Review overdue visit","")))</x:f>
@@ -6403,10 +6403,10 @@
       <x:c r="H58" s="63"/>
       <x:c r="I58" s="64"/>
       <x:c r="J58" s="62" t="str">
-        <x:f>IF(A58="","",MAX(0,H58-I58))</x:f>
+        <x:f>IF(A58="","",IF(G58="Cancelled",0,MAX(0,H58-I58)))</x:f>
       </x:c>
       <x:c r="K58" s="2" t="str">
-        <x:f>IF(A58="","",IF(J58=0,"Paid",IF(I58=0,"Unpaid","Partial")))</x:f>
+        <x:f>IF(A58="","",IF(G58="Cancelled","No charge",IF(J58=0,"Paid",IF(I58&gt;0,"Partial","Unpaid"))))</x:f>
       </x:c>
       <x:c r="L58" s="2" t="str">
         <x:f>IF(A58="","",IF(AND(G58="Completed",J58&gt;0),"Collect balance",IF(AND(G58="Scheduled",B58&lt;TODAY()),"Review overdue visit","")))</x:f>
@@ -6437,10 +6437,10 @@
       <x:c r="H59" s="63"/>
       <x:c r="I59" s="64"/>
       <x:c r="J59" s="62" t="str">
-        <x:f>IF(A59="","",MAX(0,H59-I59))</x:f>
+        <x:f>IF(A59="","",IF(G59="Cancelled",0,MAX(0,H59-I59)))</x:f>
       </x:c>
       <x:c r="K59" s="2" t="str">
-        <x:f>IF(A59="","",IF(J59=0,"Paid",IF(I59=0,"Unpaid","Partial")))</x:f>
+        <x:f>IF(A59="","",IF(G59="Cancelled","No charge",IF(J59=0,"Paid",IF(I59&gt;0,"Partial","Unpaid"))))</x:f>
       </x:c>
       <x:c r="L59" s="2" t="str">
         <x:f>IF(A59="","",IF(AND(G59="Completed",J59&gt;0),"Collect balance",IF(AND(G59="Scheduled",B59&lt;TODAY()),"Review overdue visit","")))</x:f>
@@ -6471,10 +6471,10 @@
       <x:c r="H60" s="63"/>
       <x:c r="I60" s="64"/>
       <x:c r="J60" s="62" t="str">
-        <x:f>IF(A60="","",MAX(0,H60-I60))</x:f>
+        <x:f>IF(A60="","",IF(G60="Cancelled",0,MAX(0,H60-I60)))</x:f>
       </x:c>
       <x:c r="K60" s="2" t="str">
-        <x:f>IF(A60="","",IF(J60=0,"Paid",IF(I60=0,"Unpaid","Partial")))</x:f>
+        <x:f>IF(A60="","",IF(G60="Cancelled","No charge",IF(J60=0,"Paid",IF(I60&gt;0,"Partial","Unpaid"))))</x:f>
       </x:c>
       <x:c r="L60" s="2" t="str">
         <x:f>IF(A60="","",IF(AND(G60="Completed",J60&gt;0),"Collect balance",IF(AND(G60="Scheduled",B60&lt;TODAY()),"Review overdue visit","")))</x:f>
@@ -6505,10 +6505,10 @@
       <x:c r="H61" s="63"/>
       <x:c r="I61" s="64"/>
       <x:c r="J61" s="62" t="str">
-        <x:f>IF(A61="","",MAX(0,H61-I61))</x:f>
+        <x:f>IF(A61="","",IF(G61="Cancelled",0,MAX(0,H61-I61)))</x:f>
       </x:c>
       <x:c r="K61" s="2" t="str">
-        <x:f>IF(A61="","",IF(J61=0,"Paid",IF(I61=0,"Unpaid","Partial")))</x:f>
+        <x:f>IF(A61="","",IF(G61="Cancelled","No charge",IF(J61=0,"Paid",IF(I61&gt;0,"Partial","Unpaid"))))</x:f>
       </x:c>
       <x:c r="L61" s="2" t="str">
         <x:f>IF(A61="","",IF(AND(G61="Completed",J61&gt;0),"Collect balance",IF(AND(G61="Scheduled",B61&lt;TODAY()),"Review overdue visit","")))</x:f>
@@ -6539,10 +6539,10 @@
       <x:c r="H62" s="63"/>
       <x:c r="I62" s="64"/>
       <x:c r="J62" s="62" t="str">
-        <x:f>IF(A62="","",MAX(0,H62-I62))</x:f>
+        <x:f>IF(A62="","",IF(G62="Cancelled",0,MAX(0,H62-I62)))</x:f>
       </x:c>
       <x:c r="K62" s="2" t="str">
-        <x:f>IF(A62="","",IF(J62=0,"Paid",IF(I62=0,"Unpaid","Partial")))</x:f>
+        <x:f>IF(A62="","",IF(G62="Cancelled","No charge",IF(J62=0,"Paid",IF(I62&gt;0,"Partial","Unpaid"))))</x:f>
       </x:c>
       <x:c r="L62" s="2" t="str">
         <x:f>IF(A62="","",IF(AND(G62="Completed",J62&gt;0),"Collect balance",IF(AND(G62="Scheduled",B62&lt;TODAY()),"Review overdue visit","")))</x:f>
@@ -6573,10 +6573,10 @@
       <x:c r="H63" s="63"/>
       <x:c r="I63" s="64"/>
       <x:c r="J63" s="62" t="str">
-        <x:f>IF(A63="","",MAX(0,H63-I63))</x:f>
+        <x:f>IF(A63="","",IF(G63="Cancelled",0,MAX(0,H63-I63)))</x:f>
       </x:c>
       <x:c r="K63" s="2" t="str">
-        <x:f>IF(A63="","",IF(J63=0,"Paid",IF(I63=0,"Unpaid","Partial")))</x:f>
+        <x:f>IF(A63="","",IF(G63="Cancelled","No charge",IF(J63=0,"Paid",IF(I63&gt;0,"Partial","Unpaid"))))</x:f>
       </x:c>
       <x:c r="L63" s="2" t="str">
         <x:f>IF(A63="","",IF(AND(G63="Completed",J63&gt;0),"Collect balance",IF(AND(G63="Scheduled",B63&lt;TODAY()),"Review overdue visit","")))</x:f>
@@ -6607,10 +6607,10 @@
       <x:c r="H64" s="63"/>
       <x:c r="I64" s="64"/>
       <x:c r="J64" s="62" t="str">
-        <x:f>IF(A64="","",MAX(0,H64-I64))</x:f>
+        <x:f>IF(A64="","",IF(G64="Cancelled",0,MAX(0,H64-I64)))</x:f>
       </x:c>
       <x:c r="K64" s="2" t="str">
-        <x:f>IF(A64="","",IF(J64=0,"Paid",IF(I64=0,"Unpaid","Partial")))</x:f>
+        <x:f>IF(A64="","",IF(G64="Cancelled","No charge",IF(J64=0,"Paid",IF(I64&gt;0,"Partial","Unpaid"))))</x:f>
       </x:c>
       <x:c r="L64" s="2" t="str">
         <x:f>IF(A64="","",IF(AND(G64="Completed",J64&gt;0),"Collect balance",IF(AND(G64="Scheduled",B64&lt;TODAY()),"Review overdue visit","")))</x:f>
@@ -6641,10 +6641,10 @@
       <x:c r="H65" s="63"/>
       <x:c r="I65" s="64"/>
       <x:c r="J65" s="62" t="str">
-        <x:f>IF(A65="","",MAX(0,H65-I65))</x:f>
+        <x:f>IF(A65="","",IF(G65="Cancelled",0,MAX(0,H65-I65)))</x:f>
       </x:c>
       <x:c r="K65" s="2" t="str">
-        <x:f>IF(A65="","",IF(J65=0,"Paid",IF(I65=0,"Unpaid","Partial")))</x:f>
+        <x:f>IF(A65="","",IF(G65="Cancelled","No charge",IF(J65=0,"Paid",IF(I65&gt;0,"Partial","Unpaid"))))</x:f>
       </x:c>
       <x:c r="L65" s="2" t="str">
         <x:f>IF(A65="","",IF(AND(G65="Completed",J65&gt;0),"Collect balance",IF(AND(G65="Scheduled",B65&lt;TODAY()),"Review overdue visit","")))</x:f>
@@ -6675,10 +6675,10 @@
       <x:c r="H66" s="63"/>
       <x:c r="I66" s="64"/>
       <x:c r="J66" s="62" t="str">
-        <x:f>IF(A66="","",MAX(0,H66-I66))</x:f>
+        <x:f>IF(A66="","",IF(G66="Cancelled",0,MAX(0,H66-I66)))</x:f>
       </x:c>
       <x:c r="K66" s="2" t="str">
-        <x:f>IF(A66="","",IF(J66=0,"Paid",IF(I66=0,"Unpaid","Partial")))</x:f>
+        <x:f>IF(A66="","",IF(G66="Cancelled","No charge",IF(J66=0,"Paid",IF(I66&gt;0,"Partial","Unpaid"))))</x:f>
       </x:c>
       <x:c r="L66" s="2" t="str">
         <x:f>IF(A66="","",IF(AND(G66="Completed",J66&gt;0),"Collect balance",IF(AND(G66="Scheduled",B66&lt;TODAY()),"Review overdue visit","")))</x:f>
@@ -6709,10 +6709,10 @@
       <x:c r="H67" s="63"/>
       <x:c r="I67" s="64"/>
       <x:c r="J67" s="62" t="str">
-        <x:f>IF(A67="","",MAX(0,H67-I67))</x:f>
+        <x:f>IF(A67="","",IF(G67="Cancelled",0,MAX(0,H67-I67)))</x:f>
       </x:c>
       <x:c r="K67" s="2" t="str">
-        <x:f>IF(A67="","",IF(J67=0,"Paid",IF(I67=0,"Unpaid","Partial")))</x:f>
+        <x:f>IF(A67="","",IF(G67="Cancelled","No charge",IF(J67=0,"Paid",IF(I67&gt;0,"Partial","Unpaid"))))</x:f>
       </x:c>
       <x:c r="L67" s="2" t="str">
         <x:f>IF(A67="","",IF(AND(G67="Completed",J67&gt;0),"Collect balance",IF(AND(G67="Scheduled",B67&lt;TODAY()),"Review overdue visit","")))</x:f>
@@ -6743,10 +6743,10 @@
       <x:c r="H68" s="63"/>
       <x:c r="I68" s="64"/>
       <x:c r="J68" s="62" t="str">
-        <x:f>IF(A68="","",MAX(0,H68-I68))</x:f>
+        <x:f>IF(A68="","",IF(G68="Cancelled",0,MAX(0,H68-I68)))</x:f>
       </x:c>
       <x:c r="K68" s="2" t="str">
-        <x:f>IF(A68="","",IF(J68=0,"Paid",IF(I68=0,"Unpaid","Partial")))</x:f>
+        <x:f>IF(A68="","",IF(G68="Cancelled","No charge",IF(J68=0,"Paid",IF(I68&gt;0,"Partial","Unpaid"))))</x:f>
       </x:c>
       <x:c r="L68" s="2" t="str">
         <x:f>IF(A68="","",IF(AND(G68="Completed",J68&gt;0),"Collect balance",IF(AND(G68="Scheduled",B68&lt;TODAY()),"Review overdue visit","")))</x:f>
@@ -6777,10 +6777,10 @@
       <x:c r="H69" s="63"/>
       <x:c r="I69" s="64"/>
       <x:c r="J69" s="62" t="str">
-        <x:f>IF(A69="","",MAX(0,H69-I69))</x:f>
+        <x:f>IF(A69="","",IF(G69="Cancelled",0,MAX(0,H69-I69)))</x:f>
       </x:c>
       <x:c r="K69" s="2" t="str">
-        <x:f>IF(A69="","",IF(J69=0,"Paid",IF(I69=0,"Unpaid","Partial")))</x:f>
+        <x:f>IF(A69="","",IF(G69="Cancelled","No charge",IF(J69=0,"Paid",IF(I69&gt;0,"Partial","Unpaid"))))</x:f>
       </x:c>
       <x:c r="L69" s="2" t="str">
         <x:f>IF(A69="","",IF(AND(G69="Completed",J69&gt;0),"Collect balance",IF(AND(G69="Scheduled",B69&lt;TODAY()),"Review overdue visit","")))</x:f>
@@ -6811,10 +6811,10 @@
       <x:c r="H70" s="63"/>
       <x:c r="I70" s="64"/>
       <x:c r="J70" s="62" t="str">
-        <x:f>IF(A70="","",MAX(0,H70-I70))</x:f>
+        <x:f>IF(A70="","",IF(G70="Cancelled",0,MAX(0,H70-I70)))</x:f>
       </x:c>
       <x:c r="K70" s="2" t="str">
-        <x:f>IF(A70="","",IF(J70=0,"Paid",IF(I70=0,"Unpaid","Partial")))</x:f>
+        <x:f>IF(A70="","",IF(G70="Cancelled","No charge",IF(J70=0,"Paid",IF(I70&gt;0,"Partial","Unpaid"))))</x:f>
       </x:c>
       <x:c r="L70" s="2" t="str">
         <x:f>IF(A70="","",IF(AND(G70="Completed",J70&gt;0),"Collect balance",IF(AND(G70="Scheduled",B70&lt;TODAY()),"Review overdue visit","")))</x:f>
@@ -6845,10 +6845,10 @@
       <x:c r="H71" s="63"/>
       <x:c r="I71" s="64"/>
       <x:c r="J71" s="62" t="str">
-        <x:f>IF(A71="","",MAX(0,H71-I71))</x:f>
+        <x:f>IF(A71="","",IF(G71="Cancelled",0,MAX(0,H71-I71)))</x:f>
       </x:c>
       <x:c r="K71" s="2" t="str">
-        <x:f>IF(A71="","",IF(J71=0,"Paid",IF(I71=0,"Unpaid","Partial")))</x:f>
+        <x:f>IF(A71="","",IF(G71="Cancelled","No charge",IF(J71=0,"Paid",IF(I71&gt;0,"Partial","Unpaid"))))</x:f>
       </x:c>
       <x:c r="L71" s="2" t="str">
         <x:f>IF(A71="","",IF(AND(G71="Completed",J71&gt;0),"Collect balance",IF(AND(G71="Scheduled",B71&lt;TODAY()),"Review overdue visit","")))</x:f>
@@ -6879,10 +6879,10 @@
       <x:c r="H72" s="63"/>
       <x:c r="I72" s="64"/>
       <x:c r="J72" s="62" t="str">
-        <x:f>IF(A72="","",MAX(0,H72-I72))</x:f>
+        <x:f>IF(A72="","",IF(G72="Cancelled",0,MAX(0,H72-I72)))</x:f>
       </x:c>
       <x:c r="K72" s="2" t="str">
-        <x:f>IF(A72="","",IF(J72=0,"Paid",IF(I72=0,"Unpaid","Partial")))</x:f>
+        <x:f>IF(A72="","",IF(G72="Cancelled","No charge",IF(J72=0,"Paid",IF(I72&gt;0,"Partial","Unpaid"))))</x:f>
       </x:c>
       <x:c r="L72" s="2" t="str">
         <x:f>IF(A72="","",IF(AND(G72="Completed",J72&gt;0),"Collect balance",IF(AND(G72="Scheduled",B72&lt;TODAY()),"Review overdue visit","")))</x:f>
@@ -6913,10 +6913,10 @@
       <x:c r="H73" s="63"/>
       <x:c r="I73" s="64"/>
       <x:c r="J73" s="62" t="str">
-        <x:f>IF(A73="","",MAX(0,H73-I73))</x:f>
+        <x:f>IF(A73="","",IF(G73="Cancelled",0,MAX(0,H73-I73)))</x:f>
       </x:c>
       <x:c r="K73" s="2" t="str">
-        <x:f>IF(A73="","",IF(J73=0,"Paid",IF(I73=0,"Unpaid","Partial")))</x:f>
+        <x:f>IF(A73="","",IF(G73="Cancelled","No charge",IF(J73=0,"Paid",IF(I73&gt;0,"Partial","Unpaid"))))</x:f>
       </x:c>
       <x:c r="L73" s="2" t="str">
         <x:f>IF(A73="","",IF(AND(G73="Completed",J73&gt;0),"Collect balance",IF(AND(G73="Scheduled",B73&lt;TODAY()),"Review overdue visit","")))</x:f>
@@ -6947,10 +6947,10 @@
       <x:c r="H74" s="63"/>
       <x:c r="I74" s="64"/>
       <x:c r="J74" s="62" t="str">
-        <x:f>IF(A74="","",MAX(0,H74-I74))</x:f>
+        <x:f>IF(A74="","",IF(G74="Cancelled",0,MAX(0,H74-I74)))</x:f>
       </x:c>
       <x:c r="K74" s="2" t="str">
-        <x:f>IF(A74="","",IF(J74=0,"Paid",IF(I74=0,"Unpaid","Partial")))</x:f>
+        <x:f>IF(A74="","",IF(G74="Cancelled","No charge",IF(J74=0,"Paid",IF(I74&gt;0,"Partial","Unpaid"))))</x:f>
       </x:c>
       <x:c r="L74" s="2" t="str">
         <x:f>IF(A74="","",IF(AND(G74="Completed",J74&gt;0),"Collect balance",IF(AND(G74="Scheduled",B74&lt;TODAY()),"Review overdue visit","")))</x:f>
@@ -6981,10 +6981,10 @@
       <x:c r="H75" s="63"/>
       <x:c r="I75" s="64"/>
       <x:c r="J75" s="62" t="str">
-        <x:f>IF(A75="","",MAX(0,H75-I75))</x:f>
+        <x:f>IF(A75="","",IF(G75="Cancelled",0,MAX(0,H75-I75)))</x:f>
       </x:c>
       <x:c r="K75" s="2" t="str">
-        <x:f>IF(A75="","",IF(J75=0,"Paid",IF(I75=0,"Unpaid","Partial")))</x:f>
+        <x:f>IF(A75="","",IF(G75="Cancelled","No charge",IF(J75=0,"Paid",IF(I75&gt;0,"Partial","Unpaid"))))</x:f>
       </x:c>
       <x:c r="L75" s="2" t="str">
         <x:f>IF(A75="","",IF(AND(G75="Completed",J75&gt;0),"Collect balance",IF(AND(G75="Scheduled",B75&lt;TODAY()),"Review overdue visit","")))</x:f>
@@ -7015,10 +7015,10 @@
       <x:c r="H76" s="63"/>
       <x:c r="I76" s="64"/>
       <x:c r="J76" s="62" t="str">
-        <x:f>IF(A76="","",MAX(0,H76-I76))</x:f>
+        <x:f>IF(A76="","",IF(G76="Cancelled",0,MAX(0,H76-I76)))</x:f>
       </x:c>
       <x:c r="K76" s="2" t="str">
-        <x:f>IF(A76="","",IF(J76=0,"Paid",IF(I76=0,"Unpaid","Partial")))</x:f>
+        <x:f>IF(A76="","",IF(G76="Cancelled","No charge",IF(J76=0,"Paid",IF(I76&gt;0,"Partial","Unpaid"))))</x:f>
       </x:c>
       <x:c r="L76" s="2" t="str">
         <x:f>IF(A76="","",IF(AND(G76="Completed",J76&gt;0),"Collect balance",IF(AND(G76="Scheduled",B76&lt;TODAY()),"Review overdue visit","")))</x:f>
@@ -7049,10 +7049,10 @@
       <x:c r="H77" s="63"/>
       <x:c r="I77" s="64"/>
       <x:c r="J77" s="62" t="str">
-        <x:f>IF(A77="","",MAX(0,H77-I77))</x:f>
+        <x:f>IF(A77="","",IF(G77="Cancelled",0,MAX(0,H77-I77)))</x:f>
       </x:c>
       <x:c r="K77" s="2" t="str">
-        <x:f>IF(A77="","",IF(J77=0,"Paid",IF(I77=0,"Unpaid","Partial")))</x:f>
+        <x:f>IF(A77="","",IF(G77="Cancelled","No charge",IF(J77=0,"Paid",IF(I77&gt;0,"Partial","Unpaid"))))</x:f>
       </x:c>
       <x:c r="L77" s="2" t="str">
         <x:f>IF(A77="","",IF(AND(G77="Completed",J77&gt;0),"Collect balance",IF(AND(G77="Scheduled",B77&lt;TODAY()),"Review overdue visit","")))</x:f>
@@ -7083,10 +7083,10 @@
       <x:c r="H78" s="63"/>
       <x:c r="I78" s="64"/>
       <x:c r="J78" s="62" t="str">
-        <x:f>IF(A78="","",MAX(0,H78-I78))</x:f>
+        <x:f>IF(A78="","",IF(G78="Cancelled",0,MAX(0,H78-I78)))</x:f>
       </x:c>
       <x:c r="K78" s="2" t="str">
-        <x:f>IF(A78="","",IF(J78=0,"Paid",IF(I78=0,"Unpaid","Partial")))</x:f>
+        <x:f>IF(A78="","",IF(G78="Cancelled","No charge",IF(J78=0,"Paid",IF(I78&gt;0,"Partial","Unpaid"))))</x:f>
       </x:c>
       <x:c r="L78" s="2" t="str">
         <x:f>IF(A78="","",IF(AND(G78="Completed",J78&gt;0),"Collect balance",IF(AND(G78="Scheduled",B78&lt;TODAY()),"Review overdue visit","")))</x:f>
@@ -7117,10 +7117,10 @@
       <x:c r="H79" s="63"/>
       <x:c r="I79" s="64"/>
       <x:c r="J79" s="62" t="str">
-        <x:f>IF(A79="","",MAX(0,H79-I79))</x:f>
+        <x:f>IF(A79="","",IF(G79="Cancelled",0,MAX(0,H79-I79)))</x:f>
       </x:c>
       <x:c r="K79" s="2" t="str">
-        <x:f>IF(A79="","",IF(J79=0,"Paid",IF(I79=0,"Unpaid","Partial")))</x:f>
+        <x:f>IF(A79="","",IF(G79="Cancelled","No charge",IF(J79=0,"Paid",IF(I79&gt;0,"Partial","Unpaid"))))</x:f>
       </x:c>
       <x:c r="L79" s="2" t="str">
         <x:f>IF(A79="","",IF(AND(G79="Completed",J79&gt;0),"Collect balance",IF(AND(G79="Scheduled",B79&lt;TODAY()),"Review overdue visit","")))</x:f>
@@ -7151,10 +7151,10 @@
       <x:c r="H80" s="63"/>
       <x:c r="I80" s="64"/>
       <x:c r="J80" s="62" t="str">
-        <x:f>IF(A80="","",MAX(0,H80-I80))</x:f>
+        <x:f>IF(A80="","",IF(G80="Cancelled",0,MAX(0,H80-I80)))</x:f>
       </x:c>
       <x:c r="K80" s="2" t="str">
-        <x:f>IF(A80="","",IF(J80=0,"Paid",IF(I80=0,"Unpaid","Partial")))</x:f>
+        <x:f>IF(A80="","",IF(G80="Cancelled","No charge",IF(J80=0,"Paid",IF(I80&gt;0,"Partial","Unpaid"))))</x:f>
       </x:c>
       <x:c r="L80" s="2" t="str">
         <x:f>IF(A80="","",IF(AND(G80="Completed",J80&gt;0),"Collect balance",IF(AND(G80="Scheduled",B80&lt;TODAY()),"Review overdue visit","")))</x:f>
@@ -7185,10 +7185,10 @@
       <x:c r="H81" s="63"/>
       <x:c r="I81" s="64"/>
       <x:c r="J81" s="62" t="str">
-        <x:f>IF(A81="","",MAX(0,H81-I81))</x:f>
+        <x:f>IF(A81="","",IF(G81="Cancelled",0,MAX(0,H81-I81)))</x:f>
       </x:c>
       <x:c r="K81" s="2" t="str">
-        <x:f>IF(A81="","",IF(J81=0,"Paid",IF(I81=0,"Unpaid","Partial")))</x:f>
+        <x:f>IF(A81="","",IF(G81="Cancelled","No charge",IF(J81=0,"Paid",IF(I81&gt;0,"Partial","Unpaid"))))</x:f>
       </x:c>
       <x:c r="L81" s="2" t="str">
         <x:f>IF(A81="","",IF(AND(G81="Completed",J81&gt;0),"Collect balance",IF(AND(G81="Scheduled",B81&lt;TODAY()),"Review overdue visit","")))</x:f>
@@ -7219,10 +7219,10 @@
       <x:c r="H82" s="63"/>
       <x:c r="I82" s="64"/>
       <x:c r="J82" s="62" t="str">
-        <x:f>IF(A82="","",MAX(0,H82-I82))</x:f>
+        <x:f>IF(A82="","",IF(G82="Cancelled",0,MAX(0,H82-I82)))</x:f>
       </x:c>
       <x:c r="K82" s="2" t="str">
-        <x:f>IF(A82="","",IF(J82=0,"Paid",IF(I82=0,"Unpaid","Partial")))</x:f>
+        <x:f>IF(A82="","",IF(G82="Cancelled","No charge",IF(J82=0,"Paid",IF(I82&gt;0,"Partial","Unpaid"))))</x:f>
       </x:c>
       <x:c r="L82" s="2" t="str">
         <x:f>IF(A82="","",IF(AND(G82="Completed",J82&gt;0),"Collect balance",IF(AND(G82="Scheduled",B82&lt;TODAY()),"Review overdue visit","")))</x:f>
@@ -7253,10 +7253,10 @@
       <x:c r="H83" s="63"/>
       <x:c r="I83" s="64"/>
       <x:c r="J83" s="62" t="str">
-        <x:f>IF(A83="","",MAX(0,H83-I83))</x:f>
+        <x:f>IF(A83="","",IF(G83="Cancelled",0,MAX(0,H83-I83)))</x:f>
       </x:c>
       <x:c r="K83" s="2" t="str">
-        <x:f>IF(A83="","",IF(J83=0,"Paid",IF(I83=0,"Unpaid","Partial")))</x:f>
+        <x:f>IF(A83="","",IF(G83="Cancelled","No charge",IF(J83=0,"Paid",IF(I83&gt;0,"Partial","Unpaid"))))</x:f>
       </x:c>
       <x:c r="L83" s="2" t="str">
         <x:f>IF(A83="","",IF(AND(G83="Completed",J83&gt;0),"Collect balance",IF(AND(G83="Scheduled",B83&lt;TODAY()),"Review overdue visit","")))</x:f>
@@ -7287,10 +7287,10 @@
       <x:c r="H84" s="63"/>
       <x:c r="I84" s="64"/>
       <x:c r="J84" s="62" t="str">
-        <x:f>IF(A84="","",MAX(0,H84-I84))</x:f>
+        <x:f>IF(A84="","",IF(G84="Cancelled",0,MAX(0,H84-I84)))</x:f>
       </x:c>
       <x:c r="K84" s="2" t="str">
-        <x:f>IF(A84="","",IF(J84=0,"Paid",IF(I84=0,"Unpaid","Partial")))</x:f>
+        <x:f>IF(A84="","",IF(G84="Cancelled","No charge",IF(J84=0,"Paid",IF(I84&gt;0,"Partial","Unpaid"))))</x:f>
       </x:c>
       <x:c r="L84" s="2" t="str">
         <x:f>IF(A84="","",IF(AND(G84="Completed",J84&gt;0),"Collect balance",IF(AND(G84="Scheduled",B84&lt;TODAY()),"Review overdue visit","")))</x:f>
@@ -7321,10 +7321,10 @@
       <x:c r="H85" s="63"/>
       <x:c r="I85" s="64"/>
       <x:c r="J85" s="62" t="str">
-        <x:f>IF(A85="","",MAX(0,H85-I85))</x:f>
+        <x:f>IF(A85="","",IF(G85="Cancelled",0,MAX(0,H85-I85)))</x:f>
       </x:c>
       <x:c r="K85" s="2" t="str">
-        <x:f>IF(A85="","",IF(J85=0,"Paid",IF(I85=0,"Unpaid","Partial")))</x:f>
+        <x:f>IF(A85="","",IF(G85="Cancelled","No charge",IF(J85=0,"Paid",IF(I85&gt;0,"Partial","Unpaid"))))</x:f>
       </x:c>
       <x:c r="L85" s="2" t="str">
         <x:f>IF(A85="","",IF(AND(G85="Completed",J85&gt;0),"Collect balance",IF(AND(G85="Scheduled",B85&lt;TODAY()),"Review overdue visit","")))</x:f>
@@ -7355,10 +7355,10 @@
       <x:c r="H86" s="63"/>
       <x:c r="I86" s="64"/>
       <x:c r="J86" s="62" t="str">
-        <x:f>IF(A86="","",MAX(0,H86-I86))</x:f>
+        <x:f>IF(A86="","",IF(G86="Cancelled",0,MAX(0,H86-I86)))</x:f>
       </x:c>
       <x:c r="K86" s="2" t="str">
-        <x:f>IF(A86="","",IF(J86=0,"Paid",IF(I86=0,"Unpaid","Partial")))</x:f>
+        <x:f>IF(A86="","",IF(G86="Cancelled","No charge",IF(J86=0,"Paid",IF(I86&gt;0,"Partial","Unpaid"))))</x:f>
       </x:c>
       <x:c r="L86" s="2" t="str">
         <x:f>IF(A86="","",IF(AND(G86="Completed",J86&gt;0),"Collect balance",IF(AND(G86="Scheduled",B86&lt;TODAY()),"Review overdue visit","")))</x:f>
@@ -7389,10 +7389,10 @@
       <x:c r="H87" s="63"/>
       <x:c r="I87" s="64"/>
       <x:c r="J87" s="62" t="str">
-        <x:f>IF(A87="","",MAX(0,H87-I87))</x:f>
+        <x:f>IF(A87="","",IF(G87="Cancelled",0,MAX(0,H87-I87)))</x:f>
       </x:c>
       <x:c r="K87" s="2" t="str">
-        <x:f>IF(A87="","",IF(J87=0,"Paid",IF(I87=0,"Unpaid","Partial")))</x:f>
+        <x:f>IF(A87="","",IF(G87="Cancelled","No charge",IF(J87=0,"Paid",IF(I87&gt;0,"Partial","Unpaid"))))</x:f>
       </x:c>
       <x:c r="L87" s="2" t="str">
         <x:f>IF(A87="","",IF(AND(G87="Completed",J87&gt;0),"Collect balance",IF(AND(G87="Scheduled",B87&lt;TODAY()),"Review overdue visit","")))</x:f>
@@ -7423,10 +7423,10 @@
       <x:c r="H88" s="63"/>
       <x:c r="I88" s="64"/>
       <x:c r="J88" s="62" t="str">
-        <x:f>IF(A88="","",MAX(0,H88-I88))</x:f>
+        <x:f>IF(A88="","",IF(G88="Cancelled",0,MAX(0,H88-I88)))</x:f>
       </x:c>
       <x:c r="K88" s="2" t="str">
-        <x:f>IF(A88="","",IF(J88=0,"Paid",IF(I88=0,"Unpaid","Partial")))</x:f>
+        <x:f>IF(A88="","",IF(G88="Cancelled","No charge",IF(J88=0,"Paid",IF(I88&gt;0,"Partial","Unpaid"))))</x:f>
       </x:c>
       <x:c r="L88" s="2" t="str">
         <x:f>IF(A88="","",IF(AND(G88="Completed",J88&gt;0),"Collect balance",IF(AND(G88="Scheduled",B88&lt;TODAY()),"Review overdue visit","")))</x:f>
@@ -7457,10 +7457,10 @@
       <x:c r="H89" s="63"/>
       <x:c r="I89" s="64"/>
       <x:c r="J89" s="62" t="str">
-        <x:f>IF(A89="","",MAX(0,H89-I89))</x:f>
+        <x:f>IF(A89="","",IF(G89="Cancelled",0,MAX(0,H89-I89)))</x:f>
       </x:c>
       <x:c r="K89" s="2" t="str">
-        <x:f>IF(A89="","",IF(J89=0,"Paid",IF(I89=0,"Unpaid","Partial")))</x:f>
+        <x:f>IF(A89="","",IF(G89="Cancelled","No charge",IF(J89=0,"Paid",IF(I89&gt;0,"Partial","Unpaid"))))</x:f>
       </x:c>
       <x:c r="L89" s="2" t="str">
         <x:f>IF(A89="","",IF(AND(G89="Completed",J89&gt;0),"Collect balance",IF(AND(G89="Scheduled",B89&lt;TODAY()),"Review overdue visit","")))</x:f>
@@ -7491,10 +7491,10 @@
       <x:c r="H90" s="63"/>
       <x:c r="I90" s="64"/>
       <x:c r="J90" s="62" t="str">
-        <x:f>IF(A90="","",MAX(0,H90-I90))</x:f>
+        <x:f>IF(A90="","",IF(G90="Cancelled",0,MAX(0,H90-I90)))</x:f>
       </x:c>
       <x:c r="K90" s="2" t="str">
-        <x:f>IF(A90="","",IF(J90=0,"Paid",IF(I90=0,"Unpaid","Partial")))</x:f>
+        <x:f>IF(A90="","",IF(G90="Cancelled","No charge",IF(J90=0,"Paid",IF(I90&gt;0,"Partial","Unpaid"))))</x:f>
       </x:c>
       <x:c r="L90" s="2" t="str">
         <x:f>IF(A90="","",IF(AND(G90="Completed",J90&gt;0),"Collect balance",IF(AND(G90="Scheduled",B90&lt;TODAY()),"Review overdue visit","")))</x:f>
@@ -7525,10 +7525,10 @@
       <x:c r="H91" s="63"/>
       <x:c r="I91" s="64"/>
       <x:c r="J91" s="62" t="str">
-        <x:f>IF(A91="","",MAX(0,H91-I91))</x:f>
+        <x:f>IF(A91="","",IF(G91="Cancelled",0,MAX(0,H91-I91)))</x:f>
       </x:c>
       <x:c r="K91" s="2" t="str">
-        <x:f>IF(A91="","",IF(J91=0,"Paid",IF(I91=0,"Unpaid","Partial")))</x:f>
+        <x:f>IF(A91="","",IF(G91="Cancelled","No charge",IF(J91=0,"Paid",IF(I91&gt;0,"Partial","Unpaid"))))</x:f>
       </x:c>
       <x:c r="L91" s="2" t="str">
         <x:f>IF(A91="","",IF(AND(G91="Completed",J91&gt;0),"Collect balance",IF(AND(G91="Scheduled",B91&lt;TODAY()),"Review overdue visit","")))</x:f>
@@ -7559,10 +7559,10 @@
       <x:c r="H92" s="63"/>
       <x:c r="I92" s="64"/>
       <x:c r="J92" s="62" t="str">
-        <x:f>IF(A92="","",MAX(0,H92-I92))</x:f>
+        <x:f>IF(A92="","",IF(G92="Cancelled",0,MAX(0,H92-I92)))</x:f>
       </x:c>
       <x:c r="K92" s="2" t="str">
-        <x:f>IF(A92="","",IF(J92=0,"Paid",IF(I92=0,"Unpaid","Partial")))</x:f>
+        <x:f>IF(A92="","",IF(G92="Cancelled","No charge",IF(J92=0,"Paid",IF(I92&gt;0,"Partial","Unpaid"))))</x:f>
       </x:c>
       <x:c r="L92" s="2" t="str">
         <x:f>IF(A92="","",IF(AND(G92="Completed",J92&gt;0),"Collect balance",IF(AND(G92="Scheduled",B92&lt;TODAY()),"Review overdue visit","")))</x:f>
@@ -7593,10 +7593,10 @@
       <x:c r="H93" s="63"/>
       <x:c r="I93" s="64"/>
       <x:c r="J93" s="62" t="str">
-        <x:f>IF(A93="","",MAX(0,H93-I93))</x:f>
+        <x:f>IF(A93="","",IF(G93="Cancelled",0,MAX(0,H93-I93)))</x:f>
       </x:c>
       <x:c r="K93" s="2" t="str">
-        <x:f>IF(A93="","",IF(J93=0,"Paid",IF(I93=0,"Unpaid","Partial")))</x:f>
+        <x:f>IF(A93="","",IF(G93="Cancelled","No charge",IF(J93=0,"Paid",IF(I93&gt;0,"Partial","Unpaid"))))</x:f>
       </x:c>
       <x:c r="L93" s="2" t="str">
         <x:f>IF(A93="","",IF(AND(G93="Completed",J93&gt;0),"Collect balance",IF(AND(G93="Scheduled",B93&lt;TODAY()),"Review overdue visit","")))</x:f>
@@ -7627,10 +7627,10 @@
       <x:c r="H94" s="63"/>
       <x:c r="I94" s="64"/>
       <x:c r="J94" s="62" t="str">
-        <x:f>IF(A94="","",MAX(0,H94-I94))</x:f>
+        <x:f>IF(A94="","",IF(G94="Cancelled",0,MAX(0,H94-I94)))</x:f>
       </x:c>
       <x:c r="K94" s="2" t="str">
-        <x:f>IF(A94="","",IF(J94=0,"Paid",IF(I94=0,"Unpaid","Partial")))</x:f>
+        <x:f>IF(A94="","",IF(G94="Cancelled","No charge",IF(J94=0,"Paid",IF(I94&gt;0,"Partial","Unpaid"))))</x:f>
       </x:c>
       <x:c r="L94" s="2" t="str">
         <x:f>IF(A94="","",IF(AND(G94="Completed",J94&gt;0),"Collect balance",IF(AND(G94="Scheduled",B94&lt;TODAY()),"Review overdue visit","")))</x:f>
@@ -7661,10 +7661,10 @@
       <x:c r="H95" s="63"/>
       <x:c r="I95" s="64"/>
       <x:c r="J95" s="62" t="str">
-        <x:f>IF(A95="","",MAX(0,H95-I95))</x:f>
+        <x:f>IF(A95="","",IF(G95="Cancelled",0,MAX(0,H95-I95)))</x:f>
       </x:c>
       <x:c r="K95" s="2" t="str">
-        <x:f>IF(A95="","",IF(J95=0,"Paid",IF(I95=0,"Unpaid","Partial")))</x:f>
+        <x:f>IF(A95="","",IF(G95="Cancelled","No charge",IF(J95=0,"Paid",IF(I95&gt;0,"Partial","Unpaid"))))</x:f>
       </x:c>
       <x:c r="L95" s="2" t="str">
         <x:f>IF(A95="","",IF(AND(G95="Completed",J95&gt;0),"Collect balance",IF(AND(G95="Scheduled",B95&lt;TODAY()),"Review overdue visit","")))</x:f>
@@ -7695,10 +7695,10 @@
       <x:c r="H96" s="63"/>
       <x:c r="I96" s="64"/>
       <x:c r="J96" s="62" t="str">
-        <x:f>IF(A96="","",MAX(0,H96-I96))</x:f>
+        <x:f>IF(A96="","",IF(G96="Cancelled",0,MAX(0,H96-I96)))</x:f>
       </x:c>
       <x:c r="K96" s="2" t="str">
-        <x:f>IF(A96="","",IF(J96=0,"Paid",IF(I96=0,"Unpaid","Partial")))</x:f>
+        <x:f>IF(A96="","",IF(G96="Cancelled","No charge",IF(J96=0,"Paid",IF(I96&gt;0,"Partial","Unpaid"))))</x:f>
       </x:c>
       <x:c r="L96" s="2" t="str">
         <x:f>IF(A96="","",IF(AND(G96="Completed",J96&gt;0),"Collect balance",IF(AND(G96="Scheduled",B96&lt;TODAY()),"Review overdue visit","")))</x:f>
@@ -7729,10 +7729,10 @@
       <x:c r="H97" s="63"/>
       <x:c r="I97" s="64"/>
       <x:c r="J97" s="62" t="str">
-        <x:f>IF(A97="","",MAX(0,H97-I97))</x:f>
+        <x:f>IF(A97="","",IF(G97="Cancelled",0,MAX(0,H97-I97)))</x:f>
       </x:c>
       <x:c r="K97" s="2" t="str">
-        <x:f>IF(A97="","",IF(J97=0,"Paid",IF(I97=0,"Unpaid","Partial")))</x:f>
+        <x:f>IF(A97="","",IF(G97="Cancelled","No charge",IF(J97=0,"Paid",IF(I97&gt;0,"Partial","Unpaid"))))</x:f>
       </x:c>
       <x:c r="L97" s="2" t="str">
         <x:f>IF(A97="","",IF(AND(G97="Completed",J97&gt;0),"Collect balance",IF(AND(G97="Scheduled",B97&lt;TODAY()),"Review overdue visit","")))</x:f>
@@ -7763,10 +7763,10 @@
       <x:c r="H98" s="63"/>
       <x:c r="I98" s="64"/>
       <x:c r="J98" s="62" t="str">
-        <x:f>IF(A98="","",MAX(0,H98-I98))</x:f>
+        <x:f>IF(A98="","",IF(G98="Cancelled",0,MAX(0,H98-I98)))</x:f>
       </x:c>
       <x:c r="K98" s="2" t="str">
-        <x:f>IF(A98="","",IF(J98=0,"Paid",IF(I98=0,"Unpaid","Partial")))</x:f>
+        <x:f>IF(A98="","",IF(G98="Cancelled","No charge",IF(J98=0,"Paid",IF(I98&gt;0,"Partial","Unpaid"))))</x:f>
       </x:c>
       <x:c r="L98" s="2" t="str">
         <x:f>IF(A98="","",IF(AND(G98="Completed",J98&gt;0),"Collect balance",IF(AND(G98="Scheduled",B98&lt;TODAY()),"Review overdue visit","")))</x:f>
@@ -7797,10 +7797,10 @@
       <x:c r="H99" s="63"/>
       <x:c r="I99" s="64"/>
       <x:c r="J99" s="62" t="str">
-        <x:f>IF(A99="","",MAX(0,H99-I99))</x:f>
+        <x:f>IF(A99="","",IF(G99="Cancelled",0,MAX(0,H99-I99)))</x:f>
       </x:c>
       <x:c r="K99" s="2" t="str">
-        <x:f>IF(A99="","",IF(J99=0,"Paid",IF(I99=0,"Unpaid","Partial")))</x:f>
+        <x:f>IF(A99="","",IF(G99="Cancelled","No charge",IF(J99=0,"Paid",IF(I99&gt;0,"Partial","Unpaid"))))</x:f>
       </x:c>
       <x:c r="L99" s="2" t="str">
         <x:f>IF(A99="","",IF(AND(G99="Completed",J99&gt;0),"Collect balance",IF(AND(G99="Scheduled",B99&lt;TODAY()),"Review overdue visit","")))</x:f>
@@ -7831,10 +7831,10 @@
       <x:c r="H100" s="63"/>
       <x:c r="I100" s="64"/>
       <x:c r="J100" s="62" t="str">
-        <x:f>IF(A100="","",MAX(0,H100-I100))</x:f>
+        <x:f>IF(A100="","",IF(G100="Cancelled",0,MAX(0,H100-I100)))</x:f>
       </x:c>
       <x:c r="K100" s="2" t="str">
-        <x:f>IF(A100="","",IF(J100=0,"Paid",IF(I100=0,"Unpaid","Partial")))</x:f>
+        <x:f>IF(A100="","",IF(G100="Cancelled","No charge",IF(J100=0,"Paid",IF(I100&gt;0,"Partial","Unpaid"))))</x:f>
       </x:c>
       <x:c r="L100" s="2" t="str">
         <x:f>IF(A100="","",IF(AND(G100="Completed",J100&gt;0),"Collect balance",IF(AND(G100="Scheduled",B100&lt;TODAY()),"Review overdue visit","")))</x:f>
@@ -7865,10 +7865,10 @@
       <x:c r="H101" s="63"/>
       <x:c r="I101" s="64"/>
       <x:c r="J101" s="62" t="str">
-        <x:f>IF(A101="","",MAX(0,H101-I101))</x:f>
+        <x:f>IF(A101="","",IF(G101="Cancelled",0,MAX(0,H101-I101)))</x:f>
       </x:c>
       <x:c r="K101" s="2" t="str">
-        <x:f>IF(A101="","",IF(J101=0,"Paid",IF(I101=0,"Unpaid","Partial")))</x:f>
+        <x:f>IF(A101="","",IF(G101="Cancelled","No charge",IF(J101=0,"Paid",IF(I101&gt;0,"Partial","Unpaid"))))</x:f>
       </x:c>
       <x:c r="L101" s="2" t="str">
         <x:f>IF(A101="","",IF(AND(G101="Completed",J101&gt;0),"Collect balance",IF(AND(G101="Scheduled",B101&lt;TODAY()),"Review overdue visit","")))</x:f>
@@ -7899,10 +7899,10 @@
       <x:c r="H102" s="63"/>
       <x:c r="I102" s="64"/>
       <x:c r="J102" s="62" t="str">
-        <x:f>IF(A102="","",MAX(0,H102-I102))</x:f>
+        <x:f>IF(A102="","",IF(G102="Cancelled",0,MAX(0,H102-I102)))</x:f>
       </x:c>
       <x:c r="K102" s="2" t="str">
-        <x:f>IF(A102="","",IF(J102=0,"Paid",IF(I102=0,"Unpaid","Partial")))</x:f>
+        <x:f>IF(A102="","",IF(G102="Cancelled","No charge",IF(J102=0,"Paid",IF(I102&gt;0,"Partial","Unpaid"))))</x:f>
       </x:c>
       <x:c r="L102" s="2" t="str">
         <x:f>IF(A102="","",IF(AND(G102="Completed",J102&gt;0),"Collect balance",IF(AND(G102="Scheduled",B102&lt;TODAY()),"Review overdue visit","")))</x:f>
@@ -7933,10 +7933,10 @@
       <x:c r="H103" s="63"/>
       <x:c r="I103" s="64"/>
       <x:c r="J103" s="62" t="str">
-        <x:f>IF(A103="","",MAX(0,H103-I103))</x:f>
+        <x:f>IF(A103="","",IF(G103="Cancelled",0,MAX(0,H103-I103)))</x:f>
       </x:c>
       <x:c r="K103" s="2" t="str">
-        <x:f>IF(A103="","",IF(J103=0,"Paid",IF(I103=0,"Unpaid","Partial")))</x:f>
+        <x:f>IF(A103="","",IF(G103="Cancelled","No charge",IF(J103=0,"Paid",IF(I103&gt;0,"Partial","Unpaid"))))</x:f>
       </x:c>
       <x:c r="L103" s="2" t="str">
         <x:f>IF(A103="","",IF(AND(G103="Completed",J103&gt;0),"Collect balance",IF(AND(G103="Scheduled",B103&lt;TODAY()),"Review overdue visit","")))</x:f>
@@ -7967,10 +7967,10 @@
       <x:c r="H104" s="63"/>
       <x:c r="I104" s="64"/>
       <x:c r="J104" s="62" t="str">
-        <x:f>IF(A104="","",MAX(0,H104-I104))</x:f>
+        <x:f>IF(A104="","",IF(G104="Cancelled",0,MAX(0,H104-I104)))</x:f>
       </x:c>
       <x:c r="K104" s="2" t="str">
-        <x:f>IF(A104="","",IF(J104=0,"Paid",IF(I104=0,"Unpaid","Partial")))</x:f>
+        <x:f>IF(A104="","",IF(G104="Cancelled","No charge",IF(J104=0,"Paid",IF(I104&gt;0,"Partial","Unpaid"))))</x:f>
       </x:c>
       <x:c r="L104" s="2" t="str">
         <x:f>IF(A104="","",IF(AND(G104="Completed",J104&gt;0),"Collect balance",IF(AND(G104="Scheduled",B104&lt;TODAY()),"Review overdue visit","")))</x:f>
@@ -8001,10 +8001,10 @@
       <x:c r="H105" s="63"/>
       <x:c r="I105" s="64"/>
       <x:c r="J105" s="62" t="str">
-        <x:f>IF(A105="","",MAX(0,H105-I105))</x:f>
+        <x:f>IF(A105="","",IF(G105="Cancelled",0,MAX(0,H105-I105)))</x:f>
       </x:c>
       <x:c r="K105" s="2" t="str">
-        <x:f>IF(A105="","",IF(J105=0,"Paid",IF(I105=0,"Unpaid","Partial")))</x:f>
+        <x:f>IF(A105="","",IF(G105="Cancelled","No charge",IF(J105=0,"Paid",IF(I105&gt;0,"Partial","Unpaid"))))</x:f>
       </x:c>
       <x:c r="L105" s="2" t="str">
         <x:f>IF(A105="","",IF(AND(G105="Completed",J105&gt;0),"Collect balance",IF(AND(G105="Scheduled",B105&lt;TODAY()),"Review overdue visit","")))</x:f>
@@ -8035,10 +8035,10 @@
       <x:c r="H106" s="65"/>
       <x:c r="I106" s="66"/>
       <x:c r="J106" s="62" t="str">
-        <x:f>IF(A106="","",MAX(0,H106-I106))</x:f>
+        <x:f>IF(A106="","",IF(G106="Cancelled",0,MAX(0,H106-I106)))</x:f>
       </x:c>
       <x:c r="K106" s="2" t="str">
-        <x:f>IF(A106="","",IF(J106=0,"Paid",IF(I106=0,"Unpaid","Partial")))</x:f>
+        <x:f>IF(A106="","",IF(G106="Cancelled","No charge",IF(J106=0,"Paid",IF(I106&gt;0,"Partial","Unpaid"))))</x:f>
       </x:c>
       <x:c r="L106" s="2" t="str">
         <x:f>IF(A106="","",IF(AND(G106="Completed",J106&gt;0),"Collect balance",IF(AND(G106="Scheduled",B106&lt;TODAY()),"Review overdue visit","")))</x:f>
@@ -8473,7 +8473,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbfa6c6c400f2450b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R59c22e3824fc4a8c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -11935,7 +11935,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbce7ae68804d4251"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7c54602333804e65"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -15809,7 +15809,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb7129d0579d54acd"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9c4f63edd23c4770"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -19264,7 +19264,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1fe43660fc8a47c2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R93904fc017b44bf8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -19465,10 +19465,10 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="B7" s="35" t="str">
-        <x:v>Delete all SAMPLE rows</x:v>
+        <x:v>Clear SAMPLE inputs</x:v>
       </x:c>
       <x:c r="C7" s="35" t="str">
-        <x:v>Every included record is synthetic and labeled SAMPLE.</x:v>
+        <x:v>Clear amber sample inputs; retain rows and blue formula cells. All sample records are synthetic.</x:v>
       </x:c>
       <x:c r="D7" s="35" t="str"/>
       <x:c r="E7" s="35" t="str"/>

</xml_diff>